<commit_message>
agentes ai codex y gemini
</commit_message>
<xml_diff>
--- a/docs/C2PRO_CRONOGRAMA_MAESTRO_v1.0.xlsx
+++ b/docs/C2PRO_CRONOGRAMA_MAESTRO_v1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esus_\Documents\AI\ZTWQ\c2pro\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378B0C16-DEED-4A2D-B89C-FD7C7717B502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17031C6-6E2E-443F-A7C6-4F6E8D73DA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Resumen Ejecutivo" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4233" uniqueCount="880">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4242" uniqueCount="883">
   <si>
     <t>C2Pro - Cronograma Maestro MVP Fase 1</t>
   </si>
@@ -2275,36 +2275,6 @@
 Entregable: Código Python completo del archivo locustfile.py, listo para ejecutarse con el comando locust.</t>
   </si>
   <si>
-    <t>Nombre: WBSGeneratorAgent Implementation Dominio: AI / Backend / Agents Story Points: 5 (Complejidad alta) Dependencias: CE-S2-007 (Client Wrapper), CE-S2-001 (Schemas)
-Aquí tienes el prompt optimizado para que la IA genere el código de este agente utilizando LangGraph (la tecnología de orquestación definida en el stack ).
-🚀 Prompt Optimizado
-Contexto: Estamos desarrollando el "Cerebro" de C2Pro (Fase 2 del Roadmap). Necesitamos implementar el Agente Generador de WBS (WBSGeneratorAgent). Este componente utiliza LangGraph para orquestar la llamada a Claude Sonnet 4. Su función es analizar las cláusulas de "Alcance" y "Especificaciones Técnicas" de un contrato y generar una Estructura de Desglose de Trabajo (WBS) jerárquica. El requisito crítico de negocio es la Trazabilidad Legal: El agente no solo debe inventar tareas; debe vincular cada ítem de la WBS a la clause_id específica que justifica su existencia.
-Rol: Actúa como un Senior AI Engineer experto en LangChain y LangGraph. Entiendes cómo estructurar "Chains of Thought" (Cadenas de Pensamiento) para tareas de descomposición complejas.
-Tarea: Crear el módulo agents/wbs_generator.py.
-Requisitos Técnicos:
-Tecnología: Utiliza LangGraph para definir el grafo de estado (StateGraph). Aunque por ahora sea un grafo lineal (Input -&gt; Generate -&gt; Output), prepáralo para ciclos de reflexión en el futuro.
-Input del Agente:
-Lista de objetos Clause (texto, id, tipo).
-Contexto del proyecto (tipo de obra, presupuesto total).
-System Prompt (Ingeniería de Prompts dentro del código):
-Debes redactar un System Prompt potente para Claude Sonnet.
-Instrucción de Jerarquía: Debe forzar una estructura estricta de 4 niveles:
-Proyecto (Raíz).
-Fase (Ingeniería, Procura, Construcción, etc.).
-Entregable Principal.
-Paquete de Trabajo (Accionable).
-Instrucción de Trazabilidad: "Cada ítem generado DEBE incluir el ID de la cláusula (source_clause_id) que lo menciona o requiere."
-Output Estructurado:
-Utiliza PydanticOutputParser o la capacidad de "Tool Calling" de Claude para forzar que la salida sea estrictamente una lista de objetos WBSItemCreate (definidos en tus schemas previos).
-Human-in-the-Loop (Gate 6):
-Configura el nodo final del grafo para que devuelva el estado con una flag requires_approval=True. Según el roadmap, el humano debe aprobar la WBS antes de guardarla.
-Entregable:
-Código Python con la clase WBSAgentState (TypedDict).
-La definición del nodo generador (generate_wbs_node).
-El System Prompt completo optimizado para descomposición de tareas EPC.
-La construcción del grafo compilado (workflow.compile()).</t>
-  </si>
-  <si>
     <t>novena actividad del Sprint 2.
 Esta actividad marca el cambio del Backend al Frontend/Diseño. Antes de escribir código React, necesitamos definir visualmente cómo será la interfaz, asegurando que cumplimos con la Gate 6 (Human-in-the-loop). Las vistas deben mostrar claramente las alertas de riesgo y obligar a la validación humana donde sea necesario.
 📝 Actividad 9: CE-S2-010
@@ -2613,40 +2583,6 @@
 La compilación del grafo (app = workflow.compile()).</t>
   </si>
   <si>
-    <t>Una vez que el WBSGeneratorAgent ha definido qué hay que hacer, el BOMBuilderAgent define con qué lo vamos a hacer. Este agente es crítico porque conecta el mundo técnico (Ingeniería) con el económico (Presupuesto) y el logístico (Compras).
-Según el Roadmap, este agente no solo lista materiales; debe ser capaz de inferir Lead Times (tiempos de entrega) y cruzar los datos con el presupuesto para cumplir la Regla R15 ("BOM sin partida presupuestaria").
-📝 Actividad 2: S3.5 (Sprint 3)
-Nombre: BOMBuilderAgent Implementation Dominio: AI / Backend / Supply Chain Story Points: 5 Dependencias: S3.4 (WBS), CE-S2-001 (Schemas)
-Aquí tienes el prompt optimizado para construir este agente experto en logística.
-🚀 Prompt Optimizado
-Contexto: Estamos desarrollando el BOMBuilderAgent (Bill of Materials) para C2Pro. Este agente recibe como entrada la WBS (generada en el paso anterior) y el Presupuesto Desglosado (partidas extraídas del BC3/Excel). Su misión es generar la lista de materiales, equipos y servicios necesarios para ejecutar cada paquete de trabajo de la WBS. Además, debe actuar como un planificador logístico experto: debe estimar los tiempos de suministro (lead_time_days) basándose en la naturaleza del ítem (ej. "Válvula especial" tarda más que "Cemento") para alimentar posteriormente las alertas de riesgo R14.
-Rol: Actúa como un Senior Supply Chain Architect y experto en LangGraph.
-Tarea: Crear el módulo agents/bom_builder.py.
-Requisitos del Grafo (State Machine):
-Estado (BOMAgentState):
-wbs_items: List[WBSItem] (Input)
-budget_items: List[BudgetItem] (Input)
-bom_items: List[BOMItem] (Output)
-Lógica del Nodo Generador (materializer_node):
-Iteración Inteligente: El agente no debe alucinar; debe iterar sobre los ítems "hoja" de la WBS.
-System Prompt: "Eres un Jefe de Compras experto en proyectos EPC. Para cada paquete de trabajo, deduce los materiales necesarios."
-Inferencia Logística: Para cada ítem generado, el LLM debe estimar:
-production_time_days: Tiempo de fabricación.
-transit_time_days: Tiempo de transporte (asumir internacional si es complejo).
-total_lead_time_days: Suma + buffer.
-Cruce Presupuestario (Regla R15): Debe intentar encontrar el budget_item_id que financia este material basándose en similitud de nombres/códigos con la lista de budget_items. Si no encuentra coincidencia clara, debe dejarlo null (lo cual disparará una alerta después).
-Integridad de Datos (Pydantic):
-El output debe cumplir estrictamente con el esquema BOMItemCreate definido en schemas/bom.py.
-Trazabilidad: Debe heredar el clause_id del ítem WBS padre.
-Optimización de Contexto:
-Dado que la WBS y el Presupuesto pueden ser enormes, implementa una estrategia de "Map-Reduce" o procesamiento por lotes (batches) en LangGraph para no desbordar la ventana de contexto de Claude.
-Entregable: Código Python con:
-La definición del BOMAgentState.
-La función materializer_node con la lógica de inferencia de lead times.
-El prompt del sistema especializado en Supply Chain.
-La configuración del grafo.</t>
-  </si>
-  <si>
     <t>l Motor de Coherencia (Coherence Engine).
 Este componente no es un agente de IA; es un Juez Determinístico. Mientras que los agentes anteriores (WBS/BOM) son "creativos" y probabilísticos, el Coherence Engine debe ser rígido y preciso. Su función es tomar todos los datos generados y aplicar las 10 Reglas Core definidas en el Roadmap para detectar contradicciones matemáticas, temporales o lógicas.
 Este motor alimenta directamente el Coherence Score y el Centro de Alertas.
@@ -2679,67 +2615,6 @@
 La clase base CoherenceRule.
 La clase CoherenceEngine (que itera y ejecuta todas las reglas).
 La implementación concreta de las reglas R1 y R14 como demostración.</t>
-  </si>
-  <si>
-    <t>Nombre: AlertGenerator Service Implementation Dominio: Backend / Core Logic Story Points: 3 Dependencias: S3.6 (Coherence Engine), CE-S2-002 (Schemas)
-Aquí tienes el prompt optimizado para implementar este servicio de persistencia inteligente.
-🚀 Prompt Optimizado
-Contexto: Estamos implementando el AlertGenerator para C2Pro. El CoherenceEngine nos entrega una lista cruda de violaciones detectadas cada vez que corre (ej. cada vez que se sube un documento). Si guardamos todo ciegamente, llenaremos la base de datos de duplicados cada vez que se ejecute el análisis. Este servicio debe actuar como un filtro inteligente: solo persistir alertas nuevas, actualizar la evidencia de las existentes y reabrir las que se creían resueltas pero han reaparecido (regresión).
-Rol: Actúa como un Backend Developer experto en patrones de diseño de sistemas de monitoreo y deduplicación de eventos.
-Tarea: Crear el módulo services/alerts/generator.py.
-Requisitos Técnicos:
-Input:
-project_id: UUID.
-detected_violations: Lista de objetos AlertCreate (generados por las reglas de S3.6).
-Lógica de Deduplicación (Fingerprinting):
-Genera un "Fingerprint" único para cada alerta basado en: rule_id + affected_entity_ids (ej. R1_schedule_123_contract_456).
-Escenario A (Nueva): Si no existe alerta activa con ese fingerprint -&gt; INSERT.
-Escenario B (Existente Open): Si ya existe y está open -&gt; UPDATE solo el evidence_json (por si los valores cambiaron) y updated_at. No crear duplicado.
-Escenario C (Regresión): Si existe pero estaba resolved -&gt; UPDATE status a open y añadir nota de sistema "Regresión detectada autom".
-Escenario D (Auto-resolve): (Opcional) Si una alerta abierta en BD ya no viene en la lista de detected_violations (el usuario arregló el problema), marcarla como resolved automáticamente.
-Human-in-the-Loop (Gate 6):
-Implementa la lógica de asignación automática de requires_human_review:
-SI severity es 'critical' O 'high' -&gt; True.
-SI rule_id afecta a cláusulas de penalización -&gt; True.
-ELSE -&gt; False (informativa).
-Trazabilidad y Persistencia:
-Asegura que el source_clause_id  se guarde correctamente.
-Usa transacciones de base de datos (atomic) para procesar el lote completo.
-Entregable: Código Python con la clase AlertGeneratorService y el método process_violations(project_id, violations). Incluye la lógica de generación del hash/fingerprint para deduplicación.</t>
-  </si>
-  <si>
-    <t>El Coherence Score no es un simple contador de errores. Es un KPI matemático (0-100) que debe resumir la salud del proyecto en un solo vistazo. Si el algoritmo es demasiado sensible, todos los proyectos tendrán "0" y el usuario se frustrará. Si es muy permisivo, todos tendrán "100" y no verán el valor.
-Según la especificación del Roadmap (Sección 12), debemos implementar una fórmula no lineal (sigmoide) para asegurar que el score siempre se mantenga entre 0 y 100, independientemente de cuántas alertas existan.
-📝 Actividad 5: S3.8 (Sprint 3)
-Nombre: Coherence Score v1 Implementation Dominio: Backend / Analytics / Math Story Points: 3 Dependencias: S3.7 (Alerts), CE-S2-002 (Schemas)
-Aquí tienes el prompt optimizado para implementar la lógica matemática definida en el Anexo técnico.
-🚀 Prompt Optimizado
-Contexto: Estamos implementando la lógica de cálculo del Coherence Score v1 para C2Pro. Este score es el indicador principal del Dashboard. Debe ser un entero entre 0 (Caos total) y 100 (Coherencia perfecta). No podemos usar una resta lineal simple (ej. 100 - (n_errores * puntos)) porque un proyecto grande con muchas alertas podría tener puntuación negativa. Según la especificación técnica del Roadmap, debemos usar una función de normalización (curva suave) y ponderar las alertas por severidad.
-Rol: Actúa como un Algorithm Engineer o Data Scientist con experiencia en implementación de métricas de riesgo (Scoring Models).
-Tarea: Crear el módulo services/scoring/calculator.py y services/scoring/weights.py.
-Requisitos del Algoritmo (Especificación Gate 5):
-Definición de Pesos (Weights):
-Define constantes para la "Penalización Base" según severidad:
-CRITICAL: 25 puntos.
-HIGH: 10 puntos.
-MEDIUM: 5 puntos.
-LOW: 1 punto.
-Cálculo de Penalización Bruta (Raw Penalty):
-Sumar el peso de todas las alertas abiertas.
-Refinamiento: Si hay múltiples alertas de la misma regla (ej. 50 materiales retrasados R14), aplicar un factor de "amortiguación logarítmica" para que no destruyan el score desproporcionadamente (ej. la primera cuenta 100%, la segunda 80%, etc., o simplemente agrupar por regla). Para v1, suma lineal por severidad es aceptable si normalizamos después.
-Fórmula de Normalización (0-100):
-Implementa la fórmula de decaimiento definida en el roadmap:
-Python
-# raw_penalty = suma de pesos
-# sensitivity = 50 (ajustable para calibración)
-normalized_score = 100 / (1 + (raw_penalty / sensitivity))
-final_score = int(max(0, min(100, normalized_score)))
-Breakdown (Explicabilidad):
-El usuario necesita saber por qué tiene un 65.
-Genera una lista de Top Drivers: Las 5 reglas que más penalización están aportando al cálculo, ordenadas descendentemente.
-Output:
-Objeto ScoreResult con: value (int), severity_breakdown (count por tipo), top_drivers (list) y calculated_at.
-Entregable: Código Python completo de la clase ScoreCalculator. Incluye comentarios explicando la fórmula matemática elegida.</t>
   </si>
   <si>
     <t>Parser PDF (S1.2) pertenece técnicamente a la fase de Ingesta (Sprint 1-2), anterior al Sprint 3 (Motor de Coherencia). Sin embargo, es un prerrequisito crítico para que los agentes del Sprint 3 (como el WBS Generator) tengan texto que procesar, así que tiene todo el sentido abordarla ahora si quedó pendiente o se está refinando. Usaremos el ID que indicas (CE-SE-001) para tu seguimiento.
@@ -3513,39 +3388,6 @@
 Entregable: router con las comprobaciones de conectividad asíncronas (await db.execute("SELECT 1")).</t>
   </si>
   <si>
-    <t>Esta actividad es el "Kill Switch" financiero. Sin este componente, un bucle infinito en un agente o un ataque de uso podría generarte una factura de miles de dólares en Anthropic en una sola noche.
-Cumple con la Gate 7 (Unit Economics): Debemos asegurar que el coste de la IA no supere el precio de la suscripción del cliente.
-Aquí tienes el prompt optimizado para un AI Lead / FinOps.
-📝 Actividad: CE-S4-002
-Nombre: Cost Controller &amp; Budget Guardrails Dominio: AI / FinOps Story Points: 1 Dependencias: CE-S4-001 (AI Service - donde se inyecta este control) Gate: Gate 7 (Cost Control) Prioridad: P0 (Riesgo Financiero Alto)
-🚀 Prompt Optimizado
-Contexto: Estamos implementando el módulo de Control de Costes (CostController) en apps/api/src/ai/cost_controller.py. Dado que usamos modelos potentes (Claude 3.5 Sonnet) con contextos largos (contratos de 100 páginas), el coste por llamada puede ser alto. Necesitamos un mecanismo de "Cortacircuitos" (Circuit Breaker) que actúe antes de cada llamada a la API. Este servicio debe monitorear el consumo acumulado del Tenant en el mes actual y bloquear las peticiones si exceden el presupuesto definido. Además, debe implementar el sistema de alertas progresivas definido en la Gate 7 (50%, 75%, 90%, 100%).
-Rol: Actúa como un AI Engineer con mentalidad de CFO (Chief Financial Officer).
-Tarea: Desarrollar la clase CostControllerService.
-Requisitos Técnicos:
-Configuración de Precios (Pricing Table):
-Define constantes con los precios actuales de Anthropic (por millón de tokens):
-CLAUDE_3_5_SONNET_INPUT = 3.00 (ejemplo, verificar precio real).
-CLAUDE_3_5_SONNET_OUTPUT = 15.00.
-CLAUDE_HAIKU_...
-Implementa un método calculate_cost(model: str, input_tokens: int, output_tokens: int) -&gt; float.
-Verificación de Presupuesto (check_budget_availability):
-Input: tenant_id.
-Lógica:
-Consultar el gasto acumulado del mes actual para ese tenant (puede ser una query SUM a la tabla de logs o consultar un contador en Redis si lo tenemos).
-Comparar con el monthly_budget_limit del tenant (configurado en DB, default ej. $50.00).
-Alertas:
-Si gasto &gt;= 50% y no se ha alertado -&gt; Log WARNING "Budget at 50%".
-Si gasto &gt;= 90% -&gt; Log CRITICAL "Budget Critical".
-Bloqueo:
-Si gasto &gt;= 100% -&gt; Lanzar BudgetExceededException. Esto detendrá la ejecución antes de llamar a Anthropic.
-Registro de Gasto (track_usage):
-Método que se llamará después de una ejecución exitosa para actualizar el contador acumulado en la base de datos.
-Resiliencia:
-El control de costes debe ser rápido. Si la base de datos tarda en responder el saldo, decide una estrategia de "Fail Open" (permitir paso) o "Fail Closed" (bloquear). Para este MVP, usa "Fail Closed" (seguridad financiera primero).
-Entregable: Código Python de la clase CostControllerService listo para ser inyectado en el AIService creado anteriormente</t>
-  </si>
-  <si>
     <t>Con la infraestructura lista (Health Checks) y la maquinaria pesada preparada (Celery Task Queue), es hora de abrir la puerta principal.
 El Endpoint de Subida de Documentos es el punto donde todo comienza. Aquí recibimos el archivo, validamos que no sea malicioso o demasiado grande, lo guardamos y le pasamos la "patata caliente" a la cola de tareas para no bloquear al usuario.
 📝 Actividad: CE-S3-010
@@ -3583,111 +3425,6 @@
 Entregable:  router completo, incluyendo la inyección de dependencias para el servicio de almacenamiento y la sesión de base de datos.</t>
   </si>
   <si>
-    <t>Esta actividad marca el hito de completitud del Motor de Coherencia. Hasta ahora teníamos el esqueleto y un par de reglas de ejemplo; ahora vamos a dotar al sistema de su verdadera inteligencia de negocio implementando las reglas complejas que cruzan Cronograma, Coste y Alcance.
-Estas reglas no son simples if/else; requieren lógica de conjuntos, comparaciones de fechas y cruces de datos entre entidades dispares (BOM vs Presupuesto).
-Aquí tienes el prompt optimizado para un AI Lead / Backend Developer.
-📝 Actividad: CE-S4-005
-Nombre: Implementación 8 Reglas de Coherencia Restantes (Core Logic) Dominio: Backend / Business Logic Story Points: 4 (Alta densidad lógica) Dependencias: CE-S3-006 (Engine Arch), CE-S4-003/004 (Agents Data) Gate: Gate 5 (Coherence Metric)
-🚀 Prompt Optimizado
-Contexto: Estamos completando el set de reglas del Coherence Engine en apps/api/src/coherence/rules/. Ya tenemos la clase base CoherenceRule y la estructura del ProjectContext. Ahora debemos implementar la lógica dura de las 8 reglas restantes para alcanzar el objetivo de "10 Reglas Core" del MVP. Estas reglas deben ser puras (sin I/O, operando sobre los datos en memoria del contexto) para asegurar velocidad y testabilidad.
-Rol: Actúa como un Business Logic Developer experto en gestión de proyectos (PMBOK) y algoritmos en Python.
-Tarea: Implementar las siguientes clases heredando de CoherenceRule.
-Detalle de las Reglas a Implementar:
-Reglas de Alcance y Coste:
-R2 (Cost Variance): Comparar Sum(BudgetItems.total) vs Contract.total_amount.
-Umbral: Si la diferencia es &gt; 5%, generar alerta HIGH. Si es &gt; 10%, CRITICAL.
-R15 (Unbudgeted Items - Zombie BOM): Iterar sobre BOMItems. Si bom_item.budget_item_id es None (no se encontró partida financiera), generar alerta HIGH por cada ítem huérfano. Evidencia: Nombre del material.
-Reglas de Cronograma y Dependencias:
-R12 (Dependency Violation): Para tareas vinculadas (Predecesora -&gt; Sucesora).
-Lógica: Si Successor.start_date &lt; Predecessor.end_date.
-Alerta: CRITICAL "Secuencia imposible".
-R20 (Orphan Tasks): Iterar WBSItems. Si un ítem hoja no tiene stakeholders asignados (RACI 'Responsible' vacío), alerta MEDIUM.
-Reglas de Cadena de Suministro (Logística):
-R14 (Lead Time Risk):
-Calcular: Fecha Necesidad en Sitio (del Cronograma) - Lead Time Total (del BOM Agent) = Fecha Límite Pedido.
-Lógica: Si Fecha Límite Pedido &lt; Hoy, alerta CRITICAL "Material ya retrasado".
-Otras Reglas (Compliance/Quality):
-R6 (Permitting): Si detectamos cláusulas de "Licencia" o "Permiso" en el contrato y no hay hito correspondiente en el cronograma.
-R19 (Cash Flow - Opcional simple): Si la curva de gastos mensual excede el límite de facturación (si tenemos esos datos). Si no, dejar como Pass por ahora.
-Requisitos Técnicos:
-Evidencia Estructurada (evidence_json):
-Cada regla debe retornar un diccionario exacto con los valores que fallaron.
-Ejemplo R14: {"material": "Válvula X", "needed_date": "2024-02-01", "lead_time": 45, "required_order_date": "2023-12-15", "delay_days": 20}. Esto es vital para que el Frontend explique el problema.
-Eficiencia:
-Usa sets o diccionarios (dict) para búsquedas rápidas (O(1)) de IDs. No hagas bucles anidados O(n^2) sobre listas grandes si puedes evitarlo indexando primero.
-Testing (Unitario):
-Para cada regla, crea un test unitario en tests/coherence/test_rules_impl.py con datos mockeados que fuercen el fallo y el éxito.
-Entregable: Código Python de las 8 clases (cada una en su archivo o agrupadas por dominio: schedule_rules.py, cost_rules.py, etc.) y sus tests unitarios.</t>
-  </si>
-  <si>
-    <t>ctividad: CE-S4-006
-Nombre: Integration Test Full Loop (Upload -&gt; Score) Dominio: QA / Testing Story Points: 3 Dependencias: Todo el Backend (S3 y S4) Gate: Gate 5 (System Coherence)
-🚀 Prompt Optimizado
-Contexto: Hemos completado los componentes individuales. Ahora necesitamos un Test de Integración de Sistema que valide el flujo completo desde la perspectiva del usuario ("Caja Negra" o "Caja Gris"). Este test simulará el viaje de un documento: Subida -&gt; Procesamiento Asíncrono -&gt; Cálculo de Score. El reto principal es manejar la asincronía (Polling) dentro del test y decidir qué mockear (para no gastar dinero en Anthropic en cada test run) y qué dejar real.
-Rol: Actúa como un QA Automation Engineer experto en pytest y pytest-asyncio.
-Tarea: Crear el test tests/integration/flows/test_full_scoring_loop.py.
-Requisitos Técnicos:
-Estrategia de Mocking (AI):
-NO llames a la API real de Anthropic.
-Usa unittest.mock o respx para interceptar las llamadas del AIService.
-Prepara "Canned Responses" (Respuestas enlatadas) realistas:
-Una respuesta para WBS Extraction (JSON con tareas).
-Una respuesta para Stakeholder Extraction (JSON con roles).
-El resto del sistema (DB, Celery, Reglas, Parsers) debe ser REAL.
-Flujo del Test (test_upload_and_calculate_score):
-Paso 1 (Upload): POST /projects/{id}/documents con un PDF de prueba (tests/fixtures/files/contract_sample.pdf).
-Assert: Status 202, retorna task_id.
-Paso 2 (Polling): Implementa un bucle while que llame a GET /projects/{id}/documents cada 0.5s (máximo 10s).
-Wait condition: Esperar hasta que el status sea PARSED.
-Paso 3 (Trigger Calculation): (Si no es automático) Llama al endpoint que dispara el cálculo de coherencia (o espera si es automático tras el parseo).
-Paso 4 (Validation): GET /projects/{id}/coherence-score.
-Assert: Status 200.
-Assert: score es un entero entre 0 y 100.
-Assert: breakdown contiene datos (no está vacío).
-Configuración Celery (Modo Test):
-Para evitar levantar un worker de Redis separado durante los tests, configura Celery en modo task_always_eager = True dentro del conftest.py. Esto hace que las tareas asíncronas se ejecuten síncronamente en el mismo hilo, facilitando el debugging y eliminando la necesidad de time.sleep().
-Entregable: Código Python del test de integración completo, incluyendo los mocks necesarios para simular la "inteligencia" de la IA sin coste.</t>
-  </si>
-  <si>
-    <t>Esta actividad es el Traductor de Negocio.
-Las reglas que implementamos en el paso anterior (CE-S4-005) devuelven datos crudos (ej: R14: Failed, delay=20). El usuario final no entiende de reglas; necesita un mensaje claro: "La Válvula X llegará 20 días tarde según el Lead Time".
-El AlertGenerator toma la lógica técnica y la convierte en Mensajes Accionables con hipervínculos a la fuente del problema (Trazabilidad).
-📝 Actividad: CE-S4-006
-Nombre: AlertGenerator con Evidencias Estructuradas Dominio: Backend / Business Logic Story Points: 1 Dependencias: CE-S4-005 (Rules Implementation) Gate: Gate 5 (Coherence Metric)
-🚀 Prompt Optimizado
-Contexto: Hemos ejecutado el motor de reglas y tenemos una lista de resultados (algunos PASS, otros FAIL). Necesitamos persistir los fallos como Alertas en la base de datos para mostrarlas en el Dashboard. El AlertGenerator en apps/api/src/coherence/alert_generator.py es responsable de:
-Recibir el output crudo de una regla.
-Formatear un mensaje humano legible usando plantillas (Templates).
-Vincular la alerta a los objetos afectados (ID de la tarea, ID del material) para que el usuario pueda hacer clic y navegar al problema (affected_ids).
-Vincular la alerta a la cláusula del contrato que se está violando (source_clause_id), si aplica.
-Rol: Actúa como un Product Engineer enfocado en la Explicabilidad (Explainability) del sistema.
-Tarea: Implementar la clase AlertGenerator.
-Requisitos Técnicos:
-Sistema de Plantillas (Message Templates):
-Define un diccionario de templates mapeado por rule_id.
-Ejemplo:
-Python
-TEMPLATES = {
-    "R14": "El material '{material}' tiene un Lead Time de {lead_time} días, lo que retrasa la tarea '{task_name}' en {delay_days} días.",
-    "R02": "La partida presupuestaria '{code}' excede el monto contractual en {variance_percent}%.",
-    # ... resto de reglas
-}
-Usa str.format(**evidence_json) para inyectar los datos dinámicamente.
-Generación de Objetos AlertCreate:
-El método generate(rule_result: RuleResult) -&gt; AlertCreate debe mapear:
-severity: Derivado de la regla (CRITICAL/HIGH/MEDIUM/LOW).
-title: Nombre corto de la regla.
-description: El mensaje formateado.
-evidence_json: El objeto JSON crudo (para debug o visualizaciones avanzadas).
-affected_object_ids: Lista de UUIDs (ej. ID del WBS Item, ID del BOM Item).
-source_clause_id: Si la regla detectó una cláusula específica.
-Deduplicación (Opcional pero recomendada):
-Si una regla genera 100 alertas idénticas (ej. "Falta fecha de inicio"), considera agruparlas o generar una sola alerta resumen ("100 tareas sin fecha de inicio") para no inundar al usuario. Para este MVP, genera alertas individuales pero pon un comentario TODO sobre la agrupación.
-Interface Limpia:
-El generador debe ser agnóstico de la base de datos. Solo transforma datos en memoria.
-Entregable: Código Python de la clase AlertGenerator con los templates definidos para las reglas implementadas en la actividad anterior.</t>
-  </si>
-  <si>
     <t>Esta es la pieza complementaria a la subida. Como el procesamiento es asíncrono, el Frontend necesita una forma de "preguntar" repetidamente: "¿Ya está listo? ¿Y ahora? ¿Y ahora?".
 Este endpoint soporta el patrón de Polling (o Long-Polling/Websockets en el futuro). Por ahora, un GET simple es suficiente para que el usuario vea cómo la barra de progreso avanza de "Subiendo" a "Analizando" y finalmente "Completado".
 📝 Actividad: CE-S3-011
@@ -3714,36 +3451,6 @@
 Optimizaciones:
 Añade soporte básico para paginación (skip, limit) aunque por defecto devuelva los últimos 20.
 Entregable: l endpoint list_project_documents.</t>
-  </si>
-  <si>
-    <t>Esta es la actividad que diferencia un "Juguete de IA" de una "Herramienta Profesional".
-Si el sistema dice que el proyecto va "Mal" (Score 40) pero un Project Manager experto dice que va "Bien" (Score 80), el usuario perderá la confianza en el primer minuto. La Calibración consiste en ajustar los Pesos (Weights) de cada regla para que la opinión de la máquina se alinee matemáticamente con la intuición humana.
-📝 Actividad: CE-S4-007
-Nombre: Calibración del Coherence Score (10 Reglas) Dominio: AI / Data Science Story Points: 1 Dependencias: CE-S4-005 (Reglas), CE-S2-015 (Gold Standard Dataset) Gate: Gate 5 (Quality Threshold &gt; 0.85 Correlation)
-🚀 Prompt Optimizado
-Contexto: Hemos implementado las 10 reglas de coherencia. Ahora debemos asignarles importancia relativa. ¿Qué es más grave: Un retraso de 2 días (R12) o un sobrecoste del 1% (R02)? Tenemos un Gold Standard Dataset (preparado en S2) con 20 proyectos anonimizados y su puntuación asignada por expertos humanos (0-100). Necesitamos un script que ejecute nuestro motor sobre estos proyectos, compare el resultado con la nota humana y calcule la correlación.
-Rol: Actúa como un Lead Data Scientist experto en validación de modelos.
-Tarea: Crear el script scripts/run_calibration.py.
-Requisitos Técnicos:
-Carga de Datos (Ground Truth):
-Leer un archivo calibration_dataset.json que contiene una lista de proyectos con sus datos crudos (WBS, BOM, Contrato) y su human_score.
-Batch Execution:
-Importar el CoherenceService.
-Iterar sobre cada proyecto del dataset e invocar calculate_score(project_context).
-Análisis Estadístico:
-Comparar ai_score vs human_score.
-Calcular:
-MSE (Mean Squared Error): Cuánto nos equivocamos en promedio.
-Correlación de Pearson: Qué tan bien sigue la tendencia (Objetivo &gt; 0.85).
-Ajuste de Pesos (Weight Tuning):
-El script debe cargar la configuración de pesos actual (DEFAULT_WEIGHTS).
-Modo Iterativo (Opcional pero valioso): Si puedes, implementa un pequeño bucle que ajuste ligeramente los pesos de las reglas críticas (CRITICAL vs HIGH) para intentar minimizar el MSE automáticamente (Hill Climbing simple), o simplemente imprime un reporte detallado sugiriendo qué reglas están penalizando demasiado.
-Output Gráfico:
-Generar un gráfico de dispersión (Scatter Plot) usando matplotlib o imprimir una tabla ASCII en consola mostrando la desviación por proyecto.
-Entregable: Código Python del script de calibración y un archivo de configuración weights_config.py optimizado</t>
-  </si>
-  <si>
-    <t>Esta actividad es la "Constitución" del sistema.En el software Enterprise (y más en construcción), los usuarios no confían en las "Cajas Negras". Si un Director de Proyecto ve una nota de 45/100, su primera pregunta será: "¿Por qué? ¿Cómo se calcula eso?".Este documento (scoring_methodology_v1.md) es la respuesta oficial. Debe ser lo suficientemente técnico para el CTO y lo suficientemente claro para que el equipo de Ventas pueda explicarlo al cliente.📝 Actividad: CE-S4-008Nombre: Documentar Fórmula Score Auditoría (Whitepaper Interno)Dominio: Documentation / AI GovernanceStory Points: 0.5Dependencias: CE-S4-007 (Pesos calibrados)Gate: Gate 5 (Auditability)🚀 Prompt OptimizadoContexto:Hemos calibrado el motor de IA y tenemos los pesos finales (CRITICAL, HIGH, MEDIUM, LOW).Ahora debemos "congelar" esta lógica en un documento oficial antes de lanzar la V1.Este documento servirá de base para la auditoría técnica y para responder dudas de clientes sobre la imparcialidad del algoritmo.La fórmula debe ser determinista: Mismos inputs = Mismo Score.Rol:Actúa como un Technical Writer con conocimientos de Data Science.Tarea:Crear el archivo docs/coherence_engine/scoring_methodology_v1.md.Requisitos del Contenido:Definición de la Fórmula Matemática:Documenta explícitamente cómo se llega al número final.Sugerencia de modelo: Modelo Deductivo (Score de Penalización).$$Score = 100 - \sum (Weight_i \times Count_i)$$(Con un suelo de 0, no negativos).O Modelo de Promedio Ponderado. Elige el que hayamos implementado en el código y explícalo con LaTeX.Tabla de Pesos (Weight Table):Lista los valores exactos acordados tras la calibración (S4-007).CRITICAL: (ej. -15 puntos).HIGH: (ej. -5 puntos).MEDIUM: (ej. -2 puntos).LOW: (ej. -0.5 puntos).Catálogo de Reglas V1:Lista las 10 reglas activas (R2, R6, R12, etc.) con una breve descripción de "Qué penaliza".Ejemplo: "R14 (Supply Chain): Penaliza si la fecha de pedido calculada es anterior a hoy."Justificación de Calibración:Añade una nota breve indicando que estos pesos fueron validados contra un dataset de 20 proyectos reales con una correlación de &gt;0.85 respecto al juicio experto.Control de Versiones:Encabezado con Version: 1.0, Date: 2026-01-24, Status: APPROVED.Entregable:Contenido en formato Markdown profesional, listo para ser commiteado al repositorio.</t>
   </si>
   <si>
     <t>Esta actividad consolida la gestión de documentos en una sola pieza de infraestructura API. Combina la Subida Asíncrona (que dispara a Celery), el Listado (que sirve para el Polling de estado) y el Borrado (limpieza).
@@ -3883,75 +3590,6 @@
 Idempotencia:
 Usa CREATE INDEX IF NOT EXISTS para evitar errores si la migración se corre dos veces.
 Entregable: Código SQL completo del archivo de migración.</t>
-  </si>
-  <si>
-    <t>Esta es la validación funcional definitiva. A diferencia de los tests unitarios (que prueban si una función "crachea"), estos tests prueban si la Lógica de Negocio es correcta.
-Si tenemos un proyecto de prueba diseñado específicamente para tener un "retraso en materiales", este test debe asegurar que la Regla R14 salte. Si no salta, tenemos un bug silencioso en la lógica.
-Aquí tienes el prompt para un QA Lead.
-📝 Actividad: CE-S4-015
-Nombre: Tests Integración Coherence Engine (Logic Validation) Dominio: Testing / QA Story Points: 1 Dependencias: CE-S4-005 (Reglas), CE-S2-015 (Golden Dataset) Gate: Gate 5 (Logic Correctness)
-🚀 Prompt Optimizado
-Contexto: El Motor de Coherencia es el corazón del producto. Hemos implementado 10 reglas complejas. Necesitamos asegurar que el motor detecta los problemas conocidos de forma determinista. Usaremos el Golden Dataset (proyectos JSON pre-fabricados con errores intencionales) para validar que las reglas se activan cuando deben. Ejemplo: Si el dataset project_broken_dates.json tiene una tarea que empieza antes de que acabe su predecesora, el test debe fallar si la regla R12 no genera una alerta CRITICAL.
-Rol: Actúa como un QA Automation Engineer especializado en validación de lógica de negocio.
-Tarea: Crear la suite de tests tests/integration/coherence/test_engine_logic.py.
-Requisitos Técnicos:
-Fixtures ("Casos de Laboratorio"):
-Crea o asegura la existencia de 2 fixtures JSON en tests/fixtures/scenarios/:
-scenario_perfect.json: Un proyecto coherente. Score esperado &gt; 90.
-scenario_disaster.json: Un proyecto con fechas imposibles, sin presupuesto y materiales tardíos. Score esperado &lt; 40.
-Test de Reglas Específicas:
-Test R12 (Dependencias): Carga un escenario con violación de secuencia. Ejecuta el motor.
-Assert: Existe una alerta con rule_id="R12".
-Assert: La severidad es CRITICAL.
-Test R02 (Sobrecoste): Carga escenario con Budget &gt; Contract.
-Assert: Existe alerta R02.
-Test de Estabilidad del Score:
-Ejecuta el motor sobre scenario_perfect.json.
-Assert: score &gt;= 90.
-Assert: La lista de alertas está vacía (o solo tiene LOW).
-Performance Check (Soft Real-time):
-Mide el tiempo de ejecución del calculate_score.
-Assert: Debe ser menor a 200ms para un proyecto de tamaño medio (el motor trabaja en memoria, debe ser rapidísimo).
-No Mocking Logic:
-A diferencia de los tests de API, aquí NO mockees las reglas. Queremos ejecutar la implementación real de CoherenceService sobre datos estáticos.
-Entregable: Código Python de los tests de integración usando pytest.</t>
-  </si>
-  <si>
-    <t>Esta actividad es crítica para la lógica RACI (Responsible, Accountable, Consulted, Informed).
-Si el sistema no sabe quién está trabajando en el proyecto, no puede detectar si hay tareas huérfanas (Regla R20). El StakeholderExtractorAgent debe leer las primeras páginas del contrato (donde suelen estar las "Partes Intervinientes") y extraer estructuradamente a las empresas y representantes legales.
-📝 Actividad: CE-S5-001
-Nombre: StakeholderExtractorAgent (NLP Entity Recognition) Dominio: AI / Backend Story Points: 3 Dependencias: CE-S4-001 (Base AI Service) Gate: Gate 5 (Accuracy &gt; 80%)
-🚀 Prompt Optimizado
-Contexto: Estamos construyendo el Agente de Identificación de Partes. Necesitamos que la IA lea el texto crudo del PDF (específicamente las secciones de introducción y firmas) y extraiga quiénes son los actores del proyecto. El objetivo es poblar la tabla stakeholders para luego poder cruzarla con el cronograma (ej. "¿Tiene esta tarea asignada a un responsable válido?").
-Rol: Actúa como un AI Engineer especialista en Procesamiento de Lenguaje Natural (NLP) y Prompt Engineering.
-Tarea: Implementar la clase StakeholderExtractorAgent en apps/api/src/agents/stakeholder_extractor.py.
-Requisitos Técnicos:
-Definición del System Prompt:
-Diseña un prompt para Claude 3.5 Sonnet que reciba texto legal desordenado y devuelva JSON estricto.
-Instrucciones Clave:
-"Identifica a la entidad 'Cliente' (Dueño de la obra) y 'Contratista' (Ejecutor)".
-"Extrae nombres de representantes legales y sus cargos si aparecen".
-"Ignora notarios o figuras irrelevantes para la ejecución (ej. registro mercantil)".
-Schema de Salida (JSON):
-JSON
-{
-  "stakeholders": [
-    {
-      "name": "Juan Pérez",
-      "role": "Project Manager", // o "Legal Representative"
-      "company": "Construcciones S.A.",
-      "type": "CONTRACTOR", // Enum: CLIENT, CONTRACTOR, SUBCONTRACTOR, SUPERVISION
-      "contact_email": "juan@construcciones.com" // Si existe
-    }
-  ]
-}
-Lógica del Agente:
-Heredar de la clase base BaseAgent.
-Implementar el método extract(text_chunk: str) -&gt; List[Stakeholder].
-Pre-procesamiento: El agente probablemente solo necesite las primeras 10 páginas y las últimas 5 (firmas) del contrato. No le envíes el documento entero de 200 páginas para ahorrar tokens.
-Manejo de Errores:
-Si el modelo alucina o devuelve JSON inválido, implementar un mecanismo de retry o usar el modo json_mode de la API de Anthropic para forzar la estructura.
-Entregable: Código Python de la clase StakeholderExtractorAgent y el prompt del sistema optimizado.</t>
   </si>
   <si>
     <t>Esta actividad convierte a la herramienta en un "Abogado/Project Manager Paranoico".
@@ -6118,6 +5756,377 @@
 apps/api/src/ai/graph/nodes.py (Lógica de agentes y crítico).
 apps/api/src/ai/graph/workflow.py (Definición del grafo y compilación).
 Script de prueba tests/ai/test_graph_flow.py que simule un ciclo completo con crítica negativa inicial.</t>
+  </si>
+  <si>
+    <t>Esta actividad es el "Kill Switch" financiero. Sin este componente, un bucle infinito en un agente o un ataque de uso podría generarte una factura de miles de dólares en Anthropic en una sola noche.
+Cumple con la Gate 7 (Unit Economics): Debemos asegurar que el coste de la IA no supere el precio de la suscripción del cliente.
+Aquí tienes el prompt optimizado para un AI Lead / FinOps.
+📝 Actividad: CE-S4-002
+Nombre: Cost Controller &amp; Budget Guardrails Dominio: AI / FinOps Story Points: 1 Dependencias: CE-S4-001 (AI Service - donde se inyecta este control) Gate: Gate 7 (Cost Control) Prioridad: P0 (Riesgo Financiero Alto)
+🚀 Prompt Optimizado
+Contexto: Estamos implementando el módulo de Control de Costes (CostController) en apps/api/src/ai/cost_controller.py. Dado que usamos modelos potentes (Claude 3.5 Sonnet) con contextos largos (contratos de 100 páginas), el coste por llamada puede ser alto. Necesitamos un mecanismo de "Cortacircuitos" (Circuit Breaker) que actúe antes de cada llamada a la API. Este servicio debe monitorear el consumo acumulado del Tenant en el mes actual y bloquear las peticiones si exceden el presupuesto definido. Además, debe implementar el sistema de alertas progresivas definido en la Gate 7 (50%, 75%, 90%, 100%).
+Rol: Actúa como un AI Engineer con mentalidad de CFO (Chief Financial Officer).
+Tarea: Desarrollar la clase CostControllerService.
+Requisitos Técnicos:
+Configuración de Precios (Pricing Table):
+Define constantes con los precios actuales de Anthropic (por millón de tokens):
+CLAUDE_3_5_SONNET_INPUT = 3.00 (ejemplo, verificar precio real).
+CLAUDE_3_5_SONNET_OUTPUT = 15.00.
+CLAUDE_HAIKU_...
+Implementa un método calculate_cost(model: str, input_tokens: int, output_tokens: int) -&gt; float.
+Verificación de Presupuesto (check_budget_availability):
+Input: tenant_id.
+Lógica:
+Consultar el gasto acumulado del mes actual para ese tenant (puede ser una query SUM a la tabla de logs o consultar un contador en Redis si lo tenemos).
+Comparar con el monthly_budget_limit del tenant (configurado en DB, default ej. $50.00).
+Alertas:
+Si gasto &gt;= 50% y no se ha alertado -&gt; Log WARNING "Budget at 50%".
+Si gasto &gt;= 90% -&gt; Log CRITICAL "Budget Critical".
+Bloqueo:
+Si gasto &gt;= 100% -&gt; Lanzar BudgetExceededException. Esto detendrá la ejecución antes de llamar a Anthropic.
+Registro de Gasto (track_usage):
+Método que se llamará después de una ejecución exitosa para actualizar el contador acumulado en la base de datos.
+Resiliencia:
+El control de costes debe ser rápido. Si la base de datos tarda en responder el saldo, decide una estrategia de "Fail Open" (permitir paso) o "Fail Closed" (bloquear). Para este MVP, usa "Fail Closed" (seguridad financiera primero).
+Entregable: Python de la clase CostControllerService listo para ser inyectado en el AIService creado anteriormente</t>
+  </si>
+  <si>
+    <t>Nombre: WBSGeneratorAgent Implementation Dominio: AI / Backend / Agents Story Points: 5 (Complejidad alta) Dependencias: CE-S2-007 (Client Wrapper), CE-S2-001 (Schemas)
+Aquí tienes el prompt optimizado para que la IA genere el código de este agente utilizando LangGraph (la tecnología de orquestación definida en el stack ).
+🚀 Prompt Optimizado
+Contexto: Estamos desarrollando el "Cerebro" de C2Pro (Fase 2 del Roadmap). Necesitamos implementar el Agente Generador de WBS (WBSGeneratorAgent). Este componente utiliza LangGraph para orquestar la llamada a Claude Sonnet 4. Su función es analizar las cláusulas de "Alcance" y "Especificaciones Técnicas" de un contrato y generar una Estructura de Desglose de Trabajo (WBS) jerárquica. El requisito crítico de negocio es la Trazabilidad Legal: El agente no solo debe inventar tareas; debe vincular cada ítem de la WBS a la clause_id específica que justifica su existencia.
+Rol: Actúa como un Senior AI Engineer experto en LangChain y LangGraph. Entiendes cómo estructurar "Chains of Thought" (Cadenas de Pensamiento) para tareas de descomposición complejas.
+Tarea: Crear el módulo agents/wbs_generator.py.
+Requisitos Técnicos:
+Tecnología: Utiliza LangGraph para definir el grafo de estado (StateGraph). Aunque por ahora sea un grafo lineal (Input -&gt; Generate -&gt; Output), prepáralo para ciclos de reflexión en el futuro.
+Input del Agente:
+Lista de objetos Clause (texto, id, tipo).
+Contexto del proyecto (tipo de obra, presupuesto total).
+System Prompt (Ingeniería de Prompts dentro del código):
+Debes redactar un System Prompt potente para Claude Sonnet.
+Instrucción de Jerarquía: Debe forzar una estructura estricta de 4 niveles:
+Proyecto (Raíz).
+Fase (Ingeniería, Procura, Construcción, etc.).
+Entregable Principal.
+Paquete de Trabajo (Accionable).
+Instrucción de Trazabilidad: "Cada ítem generado DEBE incluir el ID de la cláusula (source_clause_id) que lo menciona o requiere."
+Output Estructurado:
+Utiliza PydanticOutputParser o la capacidad de "Tool Calling" de Claude para forzar que la salida sea estrictamente una lista de objetos WBSItemCreate (definidos en tus schemas previos).
+Human-in-the-Loop (Gate 6):
+Configura el nodo final del grafo para que devuelva el estado con una flag requires_approval=True. Según el roadmap, el humano debe aprobar la WBS antes de guardarla.
+Entregable:
+Python con la clase WBSAgentState (TypedDict).
+La definición del nodo generador (generate_wbs_node).
+El System Prompt completo optimizado para descomposición de tareas EPC.
+La construcción del grafo compilado (workflow.compile()).</t>
+  </si>
+  <si>
+    <t>Una vez que el WBSGeneratorAgent ha definido qué hay que hacer, el BOMBuilderAgent define con qué lo vamos a hacer. Este agente es crítico porque conecta el mundo técnico (Ingeniería) con el económico (Presupuesto) y el logístico (Compras).
+Según el Roadmap, este agente no solo lista materiales; debe ser capaz de inferir Lead Times (tiempos de entrega) y cruzar los datos con el presupuesto para cumplir la Regla R15 ("BOM sin partida presupuestaria").
+📝 Actividad 2: S3.5 (Sprint 3)
+Nombre: BOMBuilderAgent Implementation Dominio: AI / Backend / Supply Chain Story Points: 5 Dependencias: S3.4 (WBS), CE-S2-001 (Schemas)
+Aquí tienes el prompt optimizado para construir este agente experto en logística.
+🚀 Prompt Optimizado
+Contexto: Estamos desarrollando el BOMBuilderAgent (Bill of Materials) para C2Pro. Este agente recibe como entrada la WBS (generada en el paso anterior) y el Presupuesto Desglosado (partidas extraídas del BC3/Excel). Su misión es generar la lista de materiales, equipos y servicios necesarios para ejecutar cada paquete de trabajo de la WBS. Además, debe actuar como un planificador logístico experto: debe estimar los tiempos de suministro (lead_time_days) basándose en la naturaleza del ítem (ej. "Válvula especial" tarda más que "Cemento") para alimentar posteriormente las alertas de riesgo R14.
+Rol: Actúa como un Senior Supply Chain Architect y experto en LangGraph.
+Tarea: Crear el módulo agents/bom_builder.py.
+Requisitos del Grafo (State Machine):
+Estado (BOMAgentState):
+wbs_items: List[WBSItem] (Input)
+budget_items: List[BudgetItem] (Input)
+bom_items: List[BOMItem] (Output)
+Lógica del Nodo Generador (materializer_node):
+Iteración Inteligente: El agente no debe alucinar; debe iterar sobre los ítems "hoja" de la WBS.
+System Prompt: "Eres un Jefe de Compras experto en proyectos EPC. Para cada paquete de trabajo, deduce los materiales necesarios."
+Inferencia Logística: Para cada ítem generado, el LLM debe estimar:
+production_time_days: Tiempo de fabricación.
+transit_time_days: Tiempo de transporte (asumir internacional si es complejo).
+total_lead_time_days: Suma + buffer.
+Cruce Presupuestario (Regla R15): Debe intentar encontrar el budget_item_id que financia este material basándose en similitud de nombres/códigos con la lista de budget_items. Si no encuentra coincidencia clara, debe dejarlo null (lo cual disparará una alerta después).
+Integridad de Datos (Pydantic):
+El output debe cumplir estrictamente con el esquema BOMItemCreate definido en schemas/bom.py.
+Trazabilidad: Debe heredar el clause_id del ítem WBS padre.
+Optimización de Contexto:
+Dado que la WBS y el Presupuesto pueden ser enormes, implementa una estrategia de "Map-Reduce" o procesamiento por lotes (batches) en LangGraph para no desbordar la ventana de contexto de Claude.
+Entregable: Python con:
+La definición del BOMAgentState.
+La función materializer_node con la lógica de inferencia de lead times.
+El prompt del sistema especializado en Supply Chain.
+La configuración del grafo.</t>
+  </si>
+  <si>
+    <t>Esta actividad marca el hito de completitud del Motor de Coherencia. Hasta ahora teníamos el esqueleto y un par de reglas de ejemplo; ahora vamos a dotar al sistema de su verdadera inteligencia de negocio implementando las reglas complejas que cruzan Cronograma, Coste y Alcance.
+Estas reglas no son simples if/else; requieren lógica de conjuntos, comparaciones de fechas y cruces de datos entre entidades dispares (BOM vs Presupuesto).
+Aquí tienes el prompt optimizado para un AI Lead / Backend Developer.
+📝 Actividad: CE-S4-005
+Nombre: Implementación 8 Reglas de Coherencia Restantes (Core Logic) Dominio: Backend / Business Logic Story Points: 4 (Alta densidad lógica) Dependencias: CE-S3-006 (Engine Arch), CE-S4-003/004 (Agents Data) Gate: Gate 5 (Coherence Metric)
+🚀 Prompt Optimizado
+Contexto: Estamos completando el set de reglas del Coherence Engine en apps/api/src/coherence/rules/. Ya tenemos la clase base CoherenceRule y la estructura del ProjectContext. Ahora debemos implementar la lógica dura de las 8 reglas restantes para alcanzar el objetivo de "10 Reglas Core" del MVP. Estas reglas deben ser puras (sin I/O, operando sobre los datos en memoria del contexto) para asegurar velocidad y testabilidad.
+Rol: Actúa como un Business Logic Developer experto en gestión de proyectos (PMBOK) y algoritmos en Python.
+Tarea: Implementar las siguientes clases heredando de CoherenceRule.
+Detalle de las Reglas a Implementar:
+Reglas de Alcance y Coste:
+R2 (Cost Variance): Comparar Sum(BudgetItems.total) vs Contract.total_amount.
+Umbral: Si la diferencia es &gt; 5%, generar alerta HIGH. Si es &gt; 10%, CRITICAL.
+R15 (Unbudgeted Items - Zombie BOM): Iterar sobre BOMItems. Si bom_item.budget_item_id es None (no se encontró partida financiera), generar alerta HIGH por cada ítem huérfano. Evidencia: Nombre del material.
+Reglas de Cronograma y Dependencias:
+R12 (Dependency Violation): Para tareas vinculadas (Predecesora -&gt; Sucesora).
+Lógica: Si Successor.start_date &lt; Predecessor.end_date.
+Alerta: CRITICAL "Secuencia imposible".
+R20 (Orphan Tasks): Iterar WBSItems. Si un ítem hoja no tiene stakeholders asignados (RACI 'Responsible' vacío), alerta MEDIUM.
+Reglas de Cadena de Suministro (Logística):
+R14 (Lead Time Risk):
+Calcular: Fecha Necesidad en Sitio (del Cronograma) - Lead Time Total (del BOM Agent) = Fecha Límite Pedido.
+Lógica: Si Fecha Límite Pedido &lt; Hoy, alerta CRITICAL "Material ya retrasado".
+Otras Reglas (Compliance/Quality):
+R6 (Permitting): Si detectamos cláusulas de "Licencia" o "Permiso" en el contrato y no hay hito correspondiente en el cronograma.
+R19 (Cash Flow - Opcional simple): Si la curva de gastos mensual excede el límite de facturación (si tenemos esos datos). Si no, dejar como Pass por ahora.
+Requisitos Técnicos:
+Evidencia Estructurada (evidence_json):
+Cada regla debe retornar un diccionario exacto con los valores que fallaron.
+Ejemplo R14: {"material": "Válvula X", "needed_date": "2024-02-01", "lead_time": 45, "required_order_date": "2023-12-15", "delay_days": 20}. Esto es vital para que el Frontend explique el problema.
+Eficiencia:
+Usa sets o diccionarios (dict) para búsquedas rápidas (O(1)) de IDs. No hagas bucles anidados O(n^2) sobre listas grandes si puedes evitarlo indexando primero.
+Testing (Unitario):
+Para cada regla, crea un test unitario en tests/coherence/test_rules_impl.py con datos mockeados que fuercen el fallo y el éxito.
+Entregable: Python de las 8 clases (cada una en su archivo o agrupadas por dominio: schedule_rules.py, cost_rules.py, etc.) y sus tests unitarios.</t>
+  </si>
+  <si>
+    <t>ctividad: CE-S4-006
+Nombre: Integration Test Full Loop (Upload -&gt; Score) Dominio: QA / Testing Story Points: 3 Dependencias: Todo el Backend (S3 y S4) Gate: Gate 5 (System Coherence)
+🚀 Prompt Optimizado
+Contexto: Hemos completado los componentes individuales. Ahora necesitamos un Test de Integración de Sistema que valide el flujo completo desde la perspectiva del usuario ("Caja Negra" o "Caja Gris"). Este test simulará el viaje de un documento: Subida -&gt; Procesamiento Asíncrono -&gt; Cálculo de Score. El reto principal es manejar la asincronía (Polling) dentro del test y decidir qué mockear (para no gastar dinero en Anthropic en cada test run) y qué dejar real.
+Rol: Actúa como un QA Automation Engineer experto en pytest y pytest-asyncio.
+Tarea: Crear el test tests/integration/flows/test_full_scoring_loop.py.
+Requisitos Técnicos:
+Estrategia de Mocking (AI):
+NO llames a la API real de Anthropic.
+Usa unittest.mock o respx para interceptar las llamadas del AIService.
+Prepara "Canned Responses" (Respuestas enlatadas) realistas:
+Una respuesta para WBS Extraction (JSON con tareas).
+Una respuesta para Stakeholder Extraction (JSON con roles).
+El resto del sistema (DB, Celery, Reglas, Parsers) debe ser REAL.
+Flujo del Test (test_upload_and_calculate_score):
+Paso 1 (Upload): POST /projects/{id}/documents con un PDF de prueba (tests/fixtures/files/contract_sample.pdf).
+Assert: Status 202, retorna task_id.
+Paso 2 (Polling): Implementa un bucle while que llame a GET /projects/{id}/documents cada 0.5s (máximo 10s).
+Wait condition: Esperar hasta que el status sea PARSED.
+Paso 3 (Trigger Calculation): (Si no es automático) Llama al endpoint que dispara el cálculo de coherencia (o espera si es automático tras el parseo).
+Paso 4 (Validation): GET /projects/{id}/coherence-score.
+Assert: Status 200.
+Assert: score es un entero entre 0 y 100.
+Assert: breakdown contiene datos (no está vacío).
+Configuración Celery (Modo Test):
+Para evitar levantar un worker de Redis separado durante los tests, configura Celery en modo task_always_eager = True dentro del conftest.py. Esto hace que las tareas asíncronas se ejecuten síncronamente en el mismo hilo, facilitando el debugging y eliminando la necesidad de time.sleep().
+Entregable: Python del test de integración completo, incluyendo los mocks necesarios para simular la "inteligencia" de la IA sin coste.</t>
+  </si>
+  <si>
+    <t>gemini luego codex</t>
+  </si>
+  <si>
+    <t>Esta actividad es crítica para la lógica RACI (Responsible, Accountable, Consulted, Informed).
+Si el sistema no sabe quién está trabajando en el proyecto, no puede detectar si hay tareas huérfanas (Regla R20). El StakeholderExtractorAgent debe leer las primeras páginas del contrato (donde suelen estar las "Partes Intervinientes") y extraer estructuradamente a las empresas y representantes legales.
+📝 Actividad: CE-S5-001
+Nombre: StakeholderExtractorAgent (NLP Entity Recognition) Dominio: AI / Backend Story Points: 3 Dependencias: CE-S4-001 (Base AI Service) Gate: Gate 5 (Accuracy &gt; 80%)
+🚀 Prompt Optimizado
+Contexto: Estamos construyendo el Agente de Identificación de Partes. Necesitamos que la IA lea el texto crudo del PDF (específicamente las secciones de introducción y firmas) y extraiga quiénes son los actores del proyecto. El objetivo es poblar la tabla stakeholders para luego poder cruzarla con el cronograma (ej. "¿Tiene esta tarea asignada a un responsable válido?").
+Rol: Actúa como un AI Engineer especialista en Procesamiento de Lenguaje Natural (NLP) y Prompt Engineering.
+Tarea: Implementar la clase StakeholderExtractorAgent en apps/api/src/agents/stakeholder_extractor.py.
+Requisitos Técnicos:
+Definición del System Prompt:
+Diseña un prompt para Claude 3.5 Sonnet que reciba texto legal desordenado y devuelva JSON estricto.
+Instrucciones Clave:
+"Identifica a la entidad 'Cliente' (Dueño de la obra) y 'Contratista' (Ejecutor)".
+"Extrae nombres de representantes legales y sus cargos si aparecen".
+"Ignora notarios o figuras irrelevantes para la ejecución (ej. registro mercantil)".
+Schema de Salida (JSON):
+JSON
+{
+  "stakeholders": [
+    {
+      "name": "Juan Pérez",
+      "role": "Project Manager", // o "Legal Representative"
+      "company": "Construcciones S.A.",
+      "type": "CONTRACTOR", // Enum: CLIENT, CONTRACTOR, SUBCONTRACTOR, SUPERVISION
+      "contact_email": "juan@construcciones.com" // Si existe
+    }
+  ]
+}
+Lógica del Agente:
+Heredar de la clase base BaseAgent.
+Implementar el método extract(text_chunk: str) -&gt; List[Stakeholder].
+Pre-procesamiento: El agente probablemente solo necesite las primeras 10 páginas y las últimas 5 (firmas) del contrato. No le envíes el documento entero de 200 páginas para ahorrar tokens.
+Manejo de Errores:
+Si el modelo alucina o devuelve JSON inválido, implementar un mecanismo de retry o usar el modo json_mode de la API de Anthropic para forzar la estructura.
+Entregable: Python de la clase StakeholderExtractorAgent y el prompt del sistema optimizado.</t>
+  </si>
+  <si>
+    <t>Nombre: AlertGenerator Service Implementation Dominio: Backend / Core Logic Story Points: 3 Dependencias: S3.6 (Coherence Engine), CE-S2-002 (Schemas)
+Aquí tienes el prompt optimizado para implementar este servicio de persistencia inteligente.
+🚀 Prompt Optimizado
+Contexto: Estamos implementando el AlertGenerator para C2Pro. El CoherenceEngine nos entrega una lista cruda de violaciones detectadas cada vez que corre (ej. cada vez que se sube un documento). Si guardamos todo ciegamente, llenaremos la base de datos de duplicados cada vez que se ejecute el análisis. Este servicio debe actuar como un filtro inteligente: solo persistir alertas nuevas, actualizar la evidencia de las existentes y reabrir las que se creían resueltas pero han reaparecido (regresión).
+Rol: Actúa como un Backend Developer experto en patrones de diseño de sistemas de monitoreo y deduplicación de eventos.
+Tarea: Crear el módulo services/alerts/generator.py.
+Requisitos Técnicos:
+Input:
+project_id: UUID.
+detected_violations: Lista de objetos AlertCreate (generados por las reglas de S3.6).
+Lógica de Deduplicación (Fingerprinting):
+Genera un "Fingerprint" único para cada alerta basado en: rule_id + affected_entity_ids (ej. R1_schedule_123_contract_456).
+Escenario A (Nueva): Si no existe alerta activa con ese fingerprint -&gt; INSERT.
+Escenario B (Existente Open): Si ya existe y está open -&gt; UPDATE solo el evidence_json (por si los valores cambiaron) y updated_at. No crear duplicado.
+Escenario C (Regresión): Si existe pero estaba resolved -&gt; UPDATE status a open y añadir nota de sistema "Regresión detectada autom".
+Escenario D (Auto-resolve): (Opcional) Si una alerta abierta en BD ya no viene en la lista de detected_violations (el usuario arregló el problema), marcarla como resolved automáticamente.
+Human-in-the-Loop (Gate 6):
+Implementa la lógica de asignación automática de requires_human_review:
+SI severity es 'critical' O 'high' -&gt; True.
+SI rule_id afecta a cláusulas de penalización -&gt; True.
+ELSE -&gt; False (informativa).
+Trazabilidad y Persistencia:
+Asegura que el source_clause_id  se guarde correctamente.
+Usa transacciones de base de datos (atomic) para procesar el lote completo.
+Entregable: Python con la clase AlertGeneratorService y el método process_violations(project_id, violations). Incluye la lógica de generación del hash/fingerprint para deduplicación.</t>
+  </si>
+  <si>
+    <t>Esta actividad es el Traductor de Negocio.
+Las reglas que implementamos en el paso anterior (CE-S4-005) devuelven datos crudos (ej: R14: Failed, delay=20). El usuario final no entiende de reglas; necesita un mensaje claro: "La Válvula X llegará 20 días tarde según el Lead Time".
+El AlertGenerator toma la lógica técnica y la convierte en Mensajes Accionables con hipervínculos a la fuente del problema (Trazabilidad).
+📝 Actividad: CE-S4-006
+Nombre: AlertGenerator con Evidencias Estructuradas Dominio: Backend / Business Logic Story Points: 1 Dependencias: CE-S4-005 (Rules Implementation) Gate: Gate 5 (Coherence Metric)
+🚀 Prompt Optimizado
+Contexto: Hemos ejecutado el motor de reglas y tenemos una lista de resultados (algunos PASS, otros FAIL). Necesitamos persistir los fallos como Alertas en la base de datos para mostrarlas en el Dashboard. El AlertGenerator en apps/api/src/coherence/alert_generator.py es responsable de:
+Recibir el output crudo de una regla.
+Formatear un mensaje humano legible usando plantillas (Templates).
+Vincular la alerta a los objetos afectados (ID de la tarea, ID del material) para que el usuario pueda hacer clic y navegar al problema (affected_ids).
+Vincular la alerta a la cláusula del contrato que se está violando (source_clause_id), si aplica.
+Rol: Actúa como un Product Engineer enfocado en la Explicabilidad (Explainability) del sistema.
+Tarea: Implementar la clase AlertGenerator.
+Requisitos Técnicos:
+Sistema de Plantillas (Message Templates):
+Define un diccionario de templates mapeado por rule_id.
+Ejemplo:
+Python
+TEMPLATES = {
+    "R14": "El material '{material}' tiene un Lead Time de {lead_time} días, lo que retrasa la tarea '{task_name}' en {delay_days} días.",
+    "R02": "La partida presupuestaria '{code}' excede el monto contractual en {variance_percent}%.",
+    # ... resto de reglas
+}
+Usa str.format(**evidence_json) para inyectar los datos dinámicamente.
+Generación de Objetos AlertCreate:
+El método generate(rule_result: RuleResult) -&gt; AlertCreate debe mapear:
+severity: Derivado de la regla (CRITICAL/HIGH/MEDIUM/LOW).
+title: Nombre corto de la regla.
+description: El mensaje formateado.
+evidence_json: El objeto JSON crudo (para debug o visualizaciones avanzadas).
+affected_object_ids: Lista de UUIDs (ej. ID del WBS Item, ID del BOM Item).
+source_clause_id: Si la regla detectó una cláusula específica.
+Deduplicación (Opcional pero recomendada):
+Si una regla genera 100 alertas idénticas (ej. "Falta fecha de inicio"), considera agruparlas o generar una sola alerta resumen ("100 tareas sin fecha de inicio") para no inundar al usuario. Para este MVP, genera alertas individuales pero pon un comentario TODO sobre la agrupación.
+Interface Limpia:
+El generador debe ser agnóstico de la base de datos. Solo transforma datos en memoria.
+Entregable: Python de la clase AlertGenerator con los templates definidos para las reglas implementadas en la actividad anterior.</t>
+  </si>
+  <si>
+    <t>estp hay que revisar, no me fio</t>
+  </si>
+  <si>
+    <t>Esta es la validación funcional definitiva. A diferencia de los tests unitarios (que prueban si una función "crachea"), estos tests prueban si la Lógica de Negocio es correcta.
+Si tenemos un proyecto de prueba diseñado específicamente para tener un "retraso en materiales", este test debe asegurar que la Regla R14 salte. Si no salta, tenemos un bug silencioso en la lógica.
+Aquí tienes el prompt para un QA Lead.
+📝 Actividad: CE-S4-015
+Nombre: Tests Integración Coherence Engine (Logic Validation) Dominio: Testing / QA Story Points: 1 Dependencias: CE-S4-005 (Reglas), CE-S2-015 (Golden Dataset) Gate: Gate 5 (Logic Correctness)
+🚀 Prompt Optimizado
+Contexto: El Motor de Coherencia es el corazón del producto. Hemos implementado 10 reglas complejas. Necesitamos asegurar que el motor detecta los problemas conocidos de forma determinista. Usaremos el Golden Dataset (proyectos JSON pre-fabricados con errores intencionales) para validar que las reglas se activan cuando deben. Ejemplo: Si el dataset project_broken_dates.json tiene una tarea que empieza antes de que acabe su predecesora, el test debe fallar si la regla R12 no genera una alerta CRITICAL.
+Rol: Actúa como un QA Automation Engineer especializado en validación de lógica de negocio.
+Tarea: Crear la suite de tests tests/integration/coherence/test_engine_logic.py.
+Requisitos Técnicos:
+Fixtures ("Casos de Laboratorio"):
+Crea o asegura la existencia de 2 fixtures JSON en tests/fixtures/scenarios/:
+scenario_perfect.json: Un proyecto coherente. Score esperado &gt; 90.
+scenario_disaster.json: Un proyecto con fechas imposibles, sin presupuesto y materiales tardíos. Score esperado &lt; 40.
+Test de Reglas Específicas:
+Test R12 (Dependencias): Carga un escenario con violación de secuencia. Ejecuta el motor.
+Assert: Existe una alerta con rule_id="R12".
+Assert: La severidad es CRITICAL.
+Test R02 (Sobrecoste): Carga escenario con Budget &gt; Contract.
+Assert: Existe alerta R02.
+Test de Estabilidad del Score:
+Ejecuta el motor sobre scenario_perfect.json.
+Assert: score &gt;= 90.
+Assert: La lista de alertas está vacía (o solo tiene LOW).
+Performance Check (Soft Real-time):
+Mide el tiempo de ejecución del calculate_score.
+Assert: Debe ser menor a 200ms para un proyecto de tamaño medio (el motor trabaja en memoria, debe ser rapidísimo).
+No Mocking Logic:
+A diferencia de los tests de API, aquí NO mockees las reglas. Queremos ejecutar la implementación real de CoherenceService sobre datos estáticos.
+Entregable: Python de los tests de integración usando pytest.</t>
+  </si>
+  <si>
+    <t>gemini y el otro codex</t>
+  </si>
+  <si>
+    <t>Esta es la actividad que diferencia un "Juguete de IA" de una "Herramienta Profesional".
+Si el sistema dice que el proyecto va "Mal" (Score 40) pero un Project Manager experto dice que va "Bien" (Score 80), el usuario perderá la confianza en el primer minuto. La Calibración consiste en ajustar los Pesos (Weights) de cada regla para que la opinión de la máquina se alinee matemáticamente con la intuición humana.
+📝 Actividad: CE-S4-007
+Nombre: Calibración del Coherence Score (10 Reglas) Dominio: AI / Data Science Story Points: 1 Dependencias: CE-S4-005 (Reglas), CE-S2-015 (Gold Standard Dataset) Gate: Gate 5 (Quality Threshold &gt; 0.85 Correlation)
+🚀 Prompt Optimizado
+Contexto: Hemos implementado las 10 reglas de coherencia. Ahora debemos asignarles importancia relativa. ¿Qué es más grave: Un retraso de 2 días (R12) o un sobrecoste del 1% (R02)? Tenemos un Gold Standard Dataset (preparado en S2) con 20 proyectos anonimizados y su puntuación asignada por expertos humanos (0-100). Necesitamos un script que ejecute nuestro motor sobre estos proyectos, compare el resultado con la nota humana y calcule la correlación.
+Rol: Actúa como un Lead Data Scientist experto en validación de modelos.
+Tarea: Crear el script scripts/run_calibration.py.
+Requisitos Técnicos:
+Carga de Datos (Ground Truth):
+Leer un archivo calibration_dataset.json que contiene una lista de proyectos con sus datos crudos (WBS, BOM, Contrato) y su human_score.
+Batch Execution:
+Importar el CoherenceService.
+Iterar sobre cada proyecto del dataset e invocar calculate_score(project_context).
+Análisis Estadístico:
+Comparar ai_score vs human_score.
+Calcular:
+MSE (Mean Squared Error): Cuánto nos equivocamos en promedio.
+Correlación de Pearson: Qué tan bien sigue la tendencia (Objetivo &gt; 0.85).
+Ajuste de Pesos (Weight Tuning):
+El script debe cargar la configuración de pesos actual (DEFAULT_WEIGHTS).
+Modo Iterativo (Opcional pero valioso): Si puedes, implementa un pequeño bucle que ajuste ligeramente los pesos de las reglas críticas (CRITICAL vs HIGH) para intentar minimizar el MSE automáticamente (Hill Climbing simple), o simplemente imprime un reporte detallado sugiriendo qué reglas están penalizando demasiado.
+Output Gráfico:
+Generar un gráfico de dispersión (Scatter Plot) usando matplotlib o imprimir una tabla ASCII en consola mostrando la desviación por proyecto.
+Entregable: Python del script de calibración y un archivo de configuración weights_config.py optimizado</t>
+  </si>
+  <si>
+    <t>El Coherence Score no es un simple contador de errores. Es un KPI matemático (0-100) que debe resumir la salud del proyecto en un solo vistazo. Si el algoritmo es demasiado sensible, todos los proyectos tendrán "0" y el usuario se frustrará. Si es muy permisivo, todos tendrán "100" y no verán el valor.
+Según la especificación del Roadmap (Sección 12), debemos implementar una fórmula no lineal (sigmoide) para asegurar que el score siempre se mantenga entre 0 y 100, independientemente de cuántas alertas existan.
+📝 Actividad 5: S3.8 (Sprint 3)
+Nombre: Coherence Score v1 Implementation Dominio: Backend / Analytics / Math Story Points: 3 Dependencias: S3.7 (Alerts), CE-S2-002 (Schemas)
+Aquí tienes el prompt optimizado para implementar la lógica matemática definida en el Anexo técnico.
+🚀 Prompt Optimizado
+Contexto: Estamos implementando la lógica de cálculo del Coherence Score v1 para C2Pro. Este score es el indicador principal del Dashboard. Debe ser un entero entre 0 (Caos total) y 100 (Coherencia perfecta). No podemos usar una resta lineal simple (ej. 100 - (n_errores * puntos)) porque un proyecto grande con muchas alertas podría tener puntuación negativa. Según la especificación técnica del Roadmap, debemos usar una función de normalización (curva suave) y ponderar las alertas por severidad.
+Rol: Actúa como un Algorithm Engineer o Data Scientist con experiencia en implementación de métricas de riesgo (Scoring Models).
+Tarea: Crear el módulo services/scoring/calculator.py y services/scoring/weights.py.
+Requisitos del Algoritmo (Especificación Gate 5):
+Definición de Pesos (Weights):
+Define constantes para la "Penalización Base" según severidad:
+CRITICAL: 25 puntos.
+HIGH: 10 puntos.
+MEDIUM: 5 puntos.
+LOW: 1 punto.
+Cálculo de Penalización Bruta (Raw Penalty):
+Sumar el peso de todas las alertas abiertas.
+Refinamiento: Si hay múltiples alertas de la misma regla (ej. 50 materiales retrasados R14), aplicar un factor de "amortiguación logarítmica" para que no destruyan el score desproporcionadamente (ej. la primera cuenta 100%, la segunda 80%, etc., o simplemente agrupar por regla). Para v1, suma lineal por severidad es aceptable si normalizamos después.
+Fórmula de Normalización (0-100):
+Implementa la fórmula de decaimiento definida en el roadmap:
+Python
+# raw_penalty = suma de pesos
+# sensitivity = 50 (ajustable para calibración)
+normalized_score = 100 / (1 + (raw_penalty / sensitivity))
+final_score = int(max(0, min(100, normalized_score)))
+Breakdown (Explicabilidad):
+El usuario necesita saber por qué tiene un 65.
+Genera una lista de Top Drivers: Las 5 reglas que más penalización están aportando al cálculo, ordenadas descendentemente.
+Output:
+Objeto ScoreResult con: value (int), severity_breakdown (count por tipo), top_drivers (list) y calculated_at.
+Entregable: Python completo de la clase ScoreCalculator. Incluye comentarios explicando la fórmula matemática elegida.</t>
+  </si>
+  <si>
+    <t>Esta actividad es la "Constitución" del sistema.En el software Enterprise (y más en construcción), los usuarios no confían en las "Cajas Negras". Si un Director de Proyecto ve una nota de 45/100, su primera pregunta será: "¿Por qué? ¿Cómo se calcula eso?".Este documento (scoring_methodology_v1.md) es la respuesta oficial. Debe ser lo suficientemente técnico para el CTO y lo suficientemente claro para que el equipo de Ventas pueda explicarlo al cliente.📝 Actividad: CE-S4-008Nombre: Documentar Fórmula Score Auditoría (Whitepaper Interno)Dominio: Documentation / AI GovernanceStory Points: 0.5Dependencias: CE-S4-007 (Pesos calibrados)Gate: Gate 5 (Auditability)🚀 Prompt OptimizadoContexto:Hemos calibrado el motor de IA y tenemos los pesos finales (CRITICAL, HIGH, MEDIUM, LOW).Ahora debemos "congelar" esta lógica en un documento oficial antes de lanzar la V1.Este documento servirá de base para la auditoría técnica y para responder dudas de clientes sobre la imparcialidad del algoritmo.La fórmula debe ser determinista: Mismos inputs = Mismo Score.Rol:Actúa como un Technical Writer con conocimientos de Data Science.Tarea:Crear el archivo docs/coherence_engine/scoring_methodology_v1.md.Requisitos del Contenido:Definición de la Fórmula Matemática:Documenta explícitamente cómo se llega al número final.Sugerencia de modelo: Modelo Deductivo (Score de Penalización).$$Score = 100 - \sum (Weight_i \times Count_i)$$(Con un suelo de 0, no negativos).O Modelo de Promedio Ponderado. Elige el que hayamos implementado en el código y explícalo con LaTeX.Tabla de Pesos (Weight Table):Lista los valores exactos acordados tras la calibración (S4-007).CRITICAL: (ej. -15 puntos).HIGH: (ej. -5 puntos).MEDIUM: (ej. -2 puntos).LOW: (ej. -0.5 puntos).Catálogo de Reglas V1:Lista las 10 reglas activas (R2, R6, R12, etc.) con una breve descripción de "Qué penaliza".Ejemplo: "R14 (Supply Chain): Penaliza si la fecha de pedido calculada es anterior a hoy."Justificación de Calibración:Añade una nota breve indicando que estos pesos fueron validados contra un dataset de 20 proyectos reales con una correlación de &gt;0.85 respecto al juicio experto.Control de Versiones:Encabezado con Version: 1.0, Date: 2026-01-24, Status: APPROVED.Entregable:Contenido en formato Markdown profesional, listo para ser commiteado al repositorio.,</t>
   </si>
 </sst>
 </file>
@@ -6330,7 +6339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6407,9 +6416,6 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -6418,6 +6424,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6733,15 +6748,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -8268,7 +8283,7 @@
         <v>ID Nombre Sprint Semana Fecha_Inicio Fecha_Fin Duracion_Dias Prioridad Estado Dominio CTO_Gate Dependencias Asignado Criterio_Aceptacion Riesgo Entregable</v>
       </c>
       <c r="W1" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="172.8" x14ac:dyDescent="0.3">
@@ -8327,14 +8342,14 @@
         <v>677</v>
       </c>
       <c r="S2" s="30" t="s">
-        <v>835</v>
+        <v>823</v>
       </c>
       <c r="V2" t="str">
         <f>A2 &amp; " " &amp; B2 &amp; " " &amp; C2 &amp; " " &amp; D2 &amp; " " &amp; E2 &amp; " " &amp; F2 &amp; " " &amp; G2 &amp; " " &amp; H2 &amp; " " &amp; I2 &amp; " " &amp; J2 &amp; " " &amp; K2 &amp; " " &amp; L2 &amp; " " &amp; M2 &amp; " " &amp; N2 &amp; " " &amp; O2 &amp; " " &amp; P2</f>
         <v>CE-S2-001 Schemas Pydantic Documents Module Sprint 2 Semana 2 2026-01-09 2026-01-10 2 P0 done Backend Gate 5 Ninguna Backend Lead Request/Response DTOs con clause_id y OpenAPI spec generada Bajo apps/api/src/modules/documents/schemas.py</v>
       </c>
       <c r="W2" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="259.2" x14ac:dyDescent="0.3">
@@ -8393,14 +8408,14 @@
         <v>677</v>
       </c>
       <c r="S3" s="30" t="s">
-        <v>829</v>
+        <v>817</v>
       </c>
       <c r="V3" t="str">
         <f t="shared" ref="V3:V84" si="0">A3 &amp; " " &amp; B3 &amp; " " &amp; C3 &amp; " " &amp; D3 &amp; " " &amp; E3 &amp; " " &amp; F3 &amp; " " &amp; G3 &amp; " " &amp; H3 &amp; " " &amp; I3 &amp; " " &amp; J3 &amp; " " &amp; K3 &amp; " " &amp; L3 &amp; " " &amp; M3 &amp; " " &amp; N3 &amp; " " &amp; O3 &amp; " " &amp; P3</f>
         <v>CE-S2-002 Schemas Pydantic Analysis Module Sprint 2 Semana 2 2026-01-09 2026-01-10 2 P0 done Backend Gate 5 Ninguna Backend Lead DTOs Alert/Analysis con evidence_json y validaciones Pydantic v2 Bajo apps/api/src/modules/analysis/schemas.py</v>
       </c>
       <c r="W3" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="28.8" x14ac:dyDescent="0.3">
@@ -8463,7 +8478,7 @@
         <v>CE-S2-003 Schemas Pydantic Stakeholders Module Sprint 2 Semana 2 2026-01-11 2026-01-11 1 P0 done Backend Gate 5 CE-S2-001 Backend Lead DTOs Stakeholder/WBS/BOM/RACI con clause_id FK Bajo apps/api/src/modules/stakeholders/schemas.py</v>
       </c>
       <c r="W4" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="28.8" x14ac:dyDescent="0.3">
@@ -8526,7 +8541,7 @@
         <v>CE-S2-004 Implementar Redis/Upstash Cache Sprint 2 Semana 2 2026-01-09 2026-01-09 1 P0 done Infrastructure Gate 7 Ninguna DevOps Cache extracciones por hash documento TTL 24h hit ratio &gt;80% Medio apps/api/src/core/cache.py</v>
       </c>
       <c r="W5" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.3">
@@ -8589,7 +8604,7 @@
         <v>CE-S2-005 Model Routing Dinámico Config Sprint 2 Semana 2 2026-01-10 2026-01-10 1 P0 done AI Gate 7 Ninguna AI Lead Config YAML routing Sonnet/Haiku por operación Bajo apps/api/src/ai/model_routing.yaml</v>
       </c>
       <c r="W6" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
@@ -8652,7 +8667,7 @@
         <v>CE-S2-006 Caché de Prompts Idénticos Sprint 2 Semana 2 2026-01-11 2026-01-11 1 P1 done AI Gate 7 CE-S2-004 AI Lead Hash SHA-256 input resultado cacheado 24h Bajo apps/api/src/ai/prompt_cache.py</v>
       </c>
       <c r="W7" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.3">
@@ -8715,7 +8730,7 @@
         <v>CE-S2-007 LLM Client Wrapper Anthropic Sprint 2 Semana 2 2026-01-11 2026-01-11 1 P0 done AI Gate 7 Ninguna AI Lead SDK retry exponential backoff logging cost tracking Medio apps/api/src/ai/llm_client.py</v>
       </c>
       <c r="W8" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="180" customHeight="1" x14ac:dyDescent="0.3">
@@ -8815,7 +8830,7 @@
 Snippet mostrando cómo añadir app.add_exception_handler(...) en el archivo main.py.</v>
       </c>
       <c r="W9" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
     </row>
     <row r="10" spans="1:23" ht="143.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8872,14 +8887,14 @@
         <v>677</v>
       </c>
       <c r="S10" s="26" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="V10" t="str">
         <f t="shared" si="0"/>
         <v>CE-S2-009 Error Handling Consistente API Sprint 2 Semana 2 2026-01-10 2026-01-10 1 P0 done Backend  Ninguna Backend Lead Excepciones custom códigos HTTP JSON estructurado Bajo apps/api/src/core/exceptions.py</v>
       </c>
       <c r="W10" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
     </row>
     <row r="11" spans="1:23" ht="120" customHeight="1" x14ac:dyDescent="0.3">
@@ -8938,14 +8953,14 @@
         <v>681</v>
       </c>
       <c r="S11" s="29" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="V11" t="str">
         <f t="shared" si="0"/>
         <v>CE-S2-010 Wireframes 6 Vistas Core Sprint 2 Semana 2 2026-01-09 2026-01-09 1 P0 done UX/UI Gate 6 Ninguna UX Designer Wireframes Dashboard/Projects/Evidence/Alerts/Stakeholders/RACI Medio docs/wireframes/</v>
       </c>
       <c r="W11" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
     </row>
     <row r="12" spans="1:23" ht="221.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8999,7 +9014,7 @@
         <v>2</v>
       </c>
       <c r="R12" s="23" t="s">
-        <v>877</v>
+        <v>865</v>
       </c>
       <c r="S12" s="29" t="s">
         <v>683</v>
@@ -9009,7 +9024,7 @@
         <v>CE-S2-011 Setup Next.js 14 + Tailwind + shadcn/ui Sprint 2 Semana 2 2026-01-10 2026-01-10 1 P0 done Frontend  Ninguna Frontend Lead Proyecto configurado componentes base app renderiza Bajo apps/web/</v>
       </c>
       <c r="W12" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="168" customHeight="1" x14ac:dyDescent="0.3">
@@ -9066,14 +9081,14 @@
         <v>677</v>
       </c>
       <c r="S13" s="28" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="V13" t="str">
         <f t="shared" si="0"/>
         <v>CE-S2-012 GitHub Actions CI Completo Sprint 2 Semana 2 2026-01-09 2026-01-09 1 P0 done DevOps  Ninguna DevOps Lint/test/build cada PR bloqueados sin CI verde Bajo .github/workflows/ci.yml</v>
       </c>
       <c r="W13" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="246" customHeight="1" x14ac:dyDescent="0.3">
@@ -9130,14 +9145,14 @@
         <v>677</v>
       </c>
       <c r="S14" s="28" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="V14" t="str">
         <f t="shared" si="0"/>
         <v>CE-S2-013 Auto-deploy Staging on Merge Main Sprint 2 Semana 2 2026-01-10 2026-01-10 0,5 P0 done DevOps  CE-S2-012 DevOps Railway + Vercel webhooks merge deploy &lt;5 min Bajo .github/workflows/deploy-staging.yml</v>
       </c>
       <c r="W14" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -9201,7 +9216,7 @@
         <v>CE-S2-014 Benchmark Baseline Endpoints Sprint 2 Semana 2 2026-01-11 2026-01-11 0,5 P1 done Performance  Ninguna Backend Lead Latencia P50/P95/P99 métricas baseline documentadas Bajo docs/performance/baseline.md</v>
       </c>
       <c r="W15" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
     </row>
     <row r="16" spans="1:23" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -9260,7 +9275,7 @@
         <v>677</v>
       </c>
       <c r="S16" s="28" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="T16" s="28" t="s">
         <v>685</v>
@@ -9270,7 +9285,7 @@
         <v>CE-S2-015 Golden Dataset v1.0 (10 proyectos) Sprint 2 Semana 2 2026-01-09 2026-01-10 2 P0 done Testing Gate 5 Ninguna QA Lead 10 proyectos sintéticos anotados README incluido Medio tests/golden/</v>
       </c>
       <c r="W16" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
     </row>
     <row r="17" spans="1:23" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -9332,14 +9347,14 @@
         <v>686</v>
       </c>
       <c r="T17" s="28" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="V17" t="str">
         <f t="shared" si="0"/>
         <v>CE-S2-016 Tests Regresión Accuracy CI Sprint 2 Semana 2 2026-01-11 2026-01-11 1 P0 done Testing Gate 5 CE-S2-015 QA Lead CI compara accuracy vs baseline falla si &lt;85% Medio tests/accuracy/</v>
       </c>
       <c r="W17" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
     </row>
     <row r="18" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -9398,17 +9413,17 @@
         <v>677</v>
       </c>
       <c r="S18" s="28" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="T18" s="28" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="V18" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-001 Parser PDF con PyMuPDF Sprint 3 Semana 3 2026-01-13 2026-01-15 3 P0 done Backend Gate 4 Ninguna Backend Lead Extracción texto posiciones offsets 10 PDFs test Medio apps/api/src/parsers/pdf_parser.py</v>
       </c>
       <c r="W18" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
     </row>
     <row r="19" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -9467,17 +9482,17 @@
         <v>677</v>
       </c>
       <c r="S19" s="28" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="T19" s="28" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="V19" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-002 Parser Excel con openpyxl Sprint 3 Semana 3 2026-01-13 2026-01-14 2 P0 done Backend Gate 4 Ninguna Backend Lead Lectura cronogramas presupuestos formatos estándar Bajo apps/api/src/parsers/excel_parser.py</v>
       </c>
       <c r="W19" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
     </row>
     <row r="20" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -9536,17 +9551,17 @@
         <v>677</v>
       </c>
       <c r="S20" s="28" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="T20" s="28" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="V20" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-003 Parser BC3 con pyfiebdc Sprint 3 Semana 3 2026-01-15 2026-01-16 2 P0 done Backend Gate 4 Ninguna Backend Lead Partidas presupuestarias españolas BC3 100% Medio apps/api/src/parsers/bc3_parser.py</v>
       </c>
       <c r="W20" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
     </row>
     <row r="21" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -9605,14 +9620,14 @@
         <v>677</v>
       </c>
       <c r="S21" s="28" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="V21" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-004 Anonymizer Service PII Sprint 3 Semana 3 2026-01-16 2026-01-17 2 P0 done Security Gate 8 CE-S3-001 Security Lead Detección hash DNI/email/teléfono/IBAN 0 PII Claude Alto apps/api/src/services/anonymizer.py</v>
       </c>
       <c r="W21" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
     </row>
     <row r="22" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -9671,18 +9686,18 @@
         <v>677</v>
       </c>
       <c r="S22" s="28" t="s">
-        <v>795</v>
+        <v>791</v>
       </c>
       <c r="V22" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-005 ClauseExtractorAgent Sprint 3 Semana 3 2026-01-15 2026-01-16 2 P0 done AI Gate 4 CE-S3-001 AI Lead Extracción cláusulas IDs estables únicos documento Alto apps/api/src/agents/clause_extractor.py</v>
       </c>
       <c r="W22" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
     </row>
     <row r="23" spans="1:23" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="36" t="s">
+      <c r="A23" s="33" t="s">
         <v>182</v>
       </c>
       <c r="B23" s="13" t="s">
@@ -9737,17 +9752,17 @@
         <v>677</v>
       </c>
       <c r="S23" s="28" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="T23" s="29" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="V23" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-006 Task Queue Celery/Redis Sprint 3 Semana 3 2026-01-13 2026-01-14 2 P0 done Infrastructure Gate 7 CE-S2-004 DevOps Jobs async parsing coherence 100 pág no bloquea Medio apps/api/src/tasks/</v>
       </c>
       <c r="W23" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
     </row>
     <row r="24" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -9806,17 +9821,17 @@
         <v>677</v>
       </c>
       <c r="S24" s="28" t="s">
-        <v>797</v>
+        <v>793</v>
       </c>
       <c r="T24" s="27" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="V24" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-007 Endpoint GET /projects/{id}/coherence-score Sprint 3 Semana 3 2026-01-14 2026-01-14 0,5 P0 done API Gate 5 CE-S2-001 Backend Lead Response schema validado score + breakdown Bajo apps/api/src/routers/projects.py</v>
       </c>
       <c r="W24" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
     </row>
     <row r="25" spans="1:23" ht="213.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -9873,17 +9888,17 @@
         <v>677</v>
       </c>
       <c r="S25" s="28" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="T25" s="27" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="V25" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-008 Endpoints CRUD /projects Sprint 3 Semana 3 2026-01-14 2026-01-15 1 P0 done API  CE-S2-001 Backend Lead List/Get/Create/Update/Delete tests integración Bajo apps/api/src/routers/projects.py</v>
       </c>
       <c r="W25" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
     </row>
     <row r="26" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -9940,20 +9955,20 @@
         <v>677</v>
       </c>
       <c r="S26" s="28" t="s">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="T26" s="28" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="U26" s="29" t="s">
-        <v>806</v>
+        <v>798</v>
       </c>
       <c r="V26" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-009 Health Check Endpoints Sprint 3 Semana 3 2026-01-13 2026-01-13 0,5 P0 en curso DevOps  Ninguna DevOps /health /ready /live UptimeRobot configurado Bajo apps/api/src/routers/health.py</v>
       </c>
       <c r="W26" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
     </row>
     <row r="27" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10012,7 +10027,7 @@
         <v>678</v>
       </c>
       <c r="S27" s="28" t="s">
-        <v>799</v>
+        <v>795</v>
       </c>
       <c r="U27" t="e" cm="1">
         <f t="array" aca="1" ref="U27" ca="1">unirtexto()</f>
@@ -10023,7 +10038,7 @@
         <v>CE-S3-010 Secrets Management GitHub Sprint 3 Semana 3 2026-01-14 2026-01-14 1 P0 done DevOps Gate 8 Ninguna DevOps Separación secrets entorno 0 secrets código Bajo .github/workflows/</v>
       </c>
       <c r="W27" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
     </row>
     <row r="28" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10077,14 +10092,14 @@
         <v>2</v>
       </c>
       <c r="S28" s="28" t="s">
-        <v>833</v>
+        <v>821</v>
       </c>
       <c r="V28" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-011 Tests Integración Parsers Sprint 3 Semana 3 2026-01-17 2026-01-17 1 P0 done Testing  CE-S3-001;CE-S3-002;CE-S3-003 QA Lead Tests archivos reales PDF/Excel/BC3 10 correctos Medio tests/integration/parsers/</v>
       </c>
       <c r="W28" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
     </row>
     <row r="29" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10140,22 +10155,22 @@
         <v>2</v>
       </c>
       <c r="R29" s="28" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="V29" t="str">
         <f t="shared" si="0"/>
         <v>CE-S3-012 Propagar clause_id a Stakeholders Sprint 3 Semana 3 2026-01-16 2026-01-16 1 P0 done Backend Gate 4 CE-S3-005 Backend Lead source_clause_id populated 100% stakeholders FK Medio apps/api/src/services/stakeholder_service.py</v>
       </c>
       <c r="W29" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
     </row>
     <row r="30" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="36" t="s">
+      <c r="A30" s="33" t="s">
         <v>211</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>843</v>
+        <v>831</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>19</v>
@@ -10176,7 +10191,7 @@
         <v>15</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="J30" s="13" t="s">
         <v>99</v>
@@ -10206,24 +10221,24 @@
         <v>678</v>
       </c>
       <c r="S30" s="28" t="s">
-        <v>711</v>
-      </c>
-      <c r="T30" s="29" t="s">
-        <v>878</v>
-      </c>
-      <c r="U30" s="24" t="s">
-        <v>879</v>
+        <v>707</v>
+      </c>
+      <c r="T30" s="28" t="s">
+        <v>866</v>
+      </c>
+      <c r="U30" s="28" t="s">
+        <v>867</v>
       </c>
       <c r="V30" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-001 opp Sprint 3 Semana 4 2026-01-20 2026-01-21 2 P0 en curso AI Gate 5 CE-S2-007 AI Lead Extracción funciona llamadas logueadas retry Alto apps/api/src/ai/ai_service.py</v>
+        <v>CE-S4-001 opp Sprint 3 Semana 4 2026-01-20 2026-01-21 2 P0 done AI Gate 5 CE-S2-007 AI Lead Extracción funciona llamadas logueadas retry Alto apps/api/src/ai/ai_service.py</v>
       </c>
       <c r="W30" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
     </row>
     <row r="31" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="36" t="s">
+      <c r="A31" s="33" t="s">
         <v>218</v>
       </c>
       <c r="B31" s="13" t="s">
@@ -10248,7 +10263,7 @@
         <v>15</v>
       </c>
       <c r="I31" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J31" s="13" t="s">
         <v>99</v>
@@ -10274,19 +10289,22 @@
       <c r="Q31" s="13">
         <v>2</v>
       </c>
-      <c r="S31" s="24" t="s">
-        <v>801</v>
+      <c r="R31" s="23" t="s">
+        <v>677</v>
+      </c>
+      <c r="S31" s="28" t="s">
+        <v>868</v>
       </c>
       <c r="V31" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-002 Cost Controller Budget Sprint 3 Semana 4 2026-01-20 2026-01-20 1 P0 Pendiente AI Gate 7 CE-S4-001 AI Lead Bloquea LLM exceder budget alertas 50/75/90/100% Alto apps/api/src/ai/cost_controller.py</v>
+        <v>CE-S4-002 Cost Controller Budget Sprint 3 Semana 4 2026-01-20 2026-01-20 1 P0 done AI Gate 7 CE-S4-001 AI Lead Bloquea LLM exceder budget alertas 50/75/90/100% Alto apps/api/src/ai/cost_controller.py</v>
       </c>
       <c r="W31" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
     </row>
     <row r="32" spans="1:23" ht="228.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="33" t="s">
         <v>222</v>
       </c>
       <c r="B32" s="13" t="s">
@@ -10311,7 +10329,7 @@
         <v>15</v>
       </c>
       <c r="I32" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J32" s="13" t="s">
         <v>99</v>
@@ -10337,22 +10355,25 @@
       <c r="Q32" s="13">
         <v>5</v>
       </c>
-      <c r="R32" s="24" t="s">
-        <v>688</v>
-      </c>
-      <c r="S32" s="24" t="s">
-        <v>698</v>
+      <c r="R32" s="23" t="s">
+        <v>677</v>
+      </c>
+      <c r="S32" s="28" t="s">
+        <v>869</v>
+      </c>
+      <c r="T32" s="28" t="s">
+        <v>697</v>
       </c>
       <c r="V32" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-003 WBSGeneratorAgent Sprint 3 Semana 4 2026-01-21 2026-01-22 2 P0 Pendiente AI Gate 5 CE-S4-001 AI Lead WBS 4 niveles contrato requires_approval=True Alto apps/api/src/agents/wbs_generator.py</v>
+        <v>CE-S4-003 WBSGeneratorAgent Sprint 3 Semana 4 2026-01-21 2026-01-22 2 P0 done AI Gate 5 CE-S4-001 AI Lead WBS 4 niveles contrato requires_approval=True Alto apps/api/src/agents/wbs_generator.py</v>
       </c>
       <c r="W32" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
     </row>
     <row r="33" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="33" t="s">
         <v>227</v>
       </c>
       <c r="B33" s="13" t="s">
@@ -10377,7 +10398,7 @@
         <v>15</v>
       </c>
       <c r="I33" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J33" s="13" t="s">
         <v>99</v>
@@ -10403,19 +10424,22 @@
       <c r="Q33" s="13">
         <v>5</v>
       </c>
-      <c r="R33" s="24" t="s">
-        <v>699</v>
+      <c r="R33" s="23" t="s">
+        <v>677</v>
+      </c>
+      <c r="S33" s="28" t="s">
+        <v>870</v>
       </c>
       <c r="V33" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-004 BOMBuilderAgent Sprint 3 Semana 4 2026-01-22 2026-01-23 2 P0 Pendiente AI Gate 5 CE-S4-001;CE-S4-003 AI Lead BOM lead times WBS contract_clause_id populated Alto apps/api/src/agents/bom_builder.py</v>
+        <v>CE-S4-004 BOMBuilderAgent Sprint 3 Semana 4 2026-01-22 2026-01-23 2 P0 done AI Gate 5 CE-S4-001;CE-S4-003 AI Lead BOM lead times WBS contract_clause_id populated Alto apps/api/src/agents/bom_builder.py</v>
       </c>
       <c r="W33" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
     </row>
     <row r="34" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="36" t="s">
+      <c r="A34" s="33" t="s">
         <v>233</v>
       </c>
       <c r="B34" s="13" t="s">
@@ -10440,7 +10464,7 @@
         <v>15</v>
       </c>
       <c r="I34" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J34" s="13" t="s">
         <v>99</v>
@@ -10466,18 +10490,21 @@
       <c r="Q34" s="13">
         <v>8</v>
       </c>
-      <c r="S34" s="24" t="s">
-        <v>803</v>
-      </c>
-      <c r="T34" s="24" t="s">
-        <v>804</v>
+      <c r="R34" s="23" t="s">
+        <v>879</v>
+      </c>
+      <c r="S34" s="28" t="s">
+        <v>871</v>
+      </c>
+      <c r="T34" s="39" t="s">
+        <v>872</v>
       </c>
       <c r="V34" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-005 Implementar 8 Reglas Coherencia Restantes Sprint 3 Semana 4 2026-01-21 2026-01-24 4 P0 Pendiente AI Gate 5 CE-S4-003;CE-S4-004 AI Lead R2/R6/R11/R12/R14/R15/R19/R20 10/10 reglas tests Alto apps/api/src/coherence/rules/</v>
+        <v>CE-S4-005 Implementar 8 Reglas Coherencia Restantes Sprint 3 Semana 4 2026-01-21 2026-01-24 4 P0 done AI Gate 5 CE-S4-003;CE-S4-004 AI Lead R2/R6/R11/R12/R14/R15/R19/R20 10/10 reglas tests Alto apps/api/src/coherence/rules/</v>
       </c>
       <c r="W34" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
     </row>
     <row r="35" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10506,7 +10533,7 @@
         <v>15</v>
       </c>
       <c r="I35" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J35" s="13" t="s">
         <v>99</v>
@@ -10532,18 +10559,21 @@
       <c r="Q35" s="13">
         <v>2</v>
       </c>
-      <c r="R35" s="24" t="s">
-        <v>701</v>
-      </c>
-      <c r="S35" s="24" t="s">
-        <v>805</v>
+      <c r="R35" s="23" t="s">
+        <v>678</v>
+      </c>
+      <c r="S35" s="28" t="s">
+        <v>875</v>
+      </c>
+      <c r="T35" s="28" t="s">
+        <v>876</v>
       </c>
       <c r="V35" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-006 AlertGenerator con Evidencias Sprint 3 Semana 4 2026-01-23 2026-01-23 1 P0 Pendiente AI Gate 5 CE-S4-005 AI Lead Alertas source_clause_id affected_ids evidence_json Medio apps/api/src/coherence/alert_generator.py</v>
+        <v>CE-S4-006 AlertGenerator con Evidencias Sprint 3 Semana 4 2026-01-23 2026-01-23 1 P0 done AI Gate 5 CE-S4-005 AI Lead Alertas source_clause_id affected_ids evidence_json Medio apps/api/src/coherence/alert_generator.py</v>
       </c>
       <c r="W35" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
     </row>
     <row r="36" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10572,7 +10602,7 @@
         <v>15</v>
       </c>
       <c r="I36" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J36" s="13" t="s">
         <v>99</v>
@@ -10598,18 +10628,21 @@
       <c r="Q36" s="13">
         <v>2</v>
       </c>
-      <c r="R36" s="24" t="s">
-        <v>702</v>
-      </c>
-      <c r="S36" s="24" t="s">
-        <v>807</v>
+      <c r="R36" s="23" t="s">
+        <v>678</v>
+      </c>
+      <c r="S36" s="28" t="s">
+        <v>881</v>
+      </c>
+      <c r="T36" s="28" t="s">
+        <v>880</v>
       </c>
       <c r="V36" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-007 Calibrar Coherence Score 10 Reglas Sprint 3 Semana 4 2026-01-24 2026-01-24 1 P0 Pendiente AI Gate 5 CE-S4-005;CE-S2-015 AI Lead Score correlaciona &gt;0.85 evaluación experta Alto scripts/run_calibration.py</v>
+        <v>CE-S4-007 Calibrar Coherence Score 10 Reglas Sprint 3 Semana 4 2026-01-24 2026-01-24 1 P0 done AI Gate 5 CE-S4-005;CE-S2-015 AI Lead Score correlaciona &gt;0.85 evaluación experta Alto scripts/run_calibration.py</v>
       </c>
       <c r="W36" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
     </row>
     <row r="37" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10638,7 +10671,7 @@
         <v>15</v>
       </c>
       <c r="I37" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J37" s="13" t="s">
         <v>250</v>
@@ -10664,15 +10697,18 @@
       <c r="Q37" s="13">
         <v>1</v>
       </c>
-      <c r="S37" s="24" t="s">
-        <v>808</v>
+      <c r="R37" s="23" t="s">
+        <v>678</v>
+      </c>
+      <c r="S37" s="28" t="s">
+        <v>882</v>
       </c>
       <c r="V37" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-008 Documentar Fórmula Score Auditoría Sprint 3 Semana 4 2026-01-24 2026-01-24 0,5 P0 Pendiente Documentation Gate 5 CE-S4-007 AI Lead scoring_methodology_v1.md pesos finales CTO aprueba Bajo docs/coherence_engine/scoring_methodology_v1.md</v>
+        <v>CE-S4-008 Documentar Fórmula Score Auditoría Sprint 3 Semana 4 2026-01-24 2026-01-24 0,5 P0 done Documentation Gate 5 CE-S4-007 AI Lead scoring_methodology_v1.md pesos finales CTO aprueba Bajo docs/coherence_engine/scoring_methodology_v1.md</v>
       </c>
       <c r="W37" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
     </row>
     <row r="38" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10731,14 +10767,14 @@
         <v>677</v>
       </c>
       <c r="S38" s="28" t="s">
-        <v>876</v>
+        <v>864</v>
       </c>
       <c r="V38" t="str">
         <f t="shared" si="0"/>
         <v>CE-S4-009 Endpoints /projects/{id}/alerts Sprint 3 Semana 4 2026-01-22 2026-01-22 1 P0 done API Gate 4 CE-S2-001 Backend Lead List filtros/Get/Resolve incluye source_clause_id Bajo apps/api/src/routers/alerts.py</v>
       </c>
       <c r="W38" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
     </row>
     <row r="39" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10767,7 +10803,7 @@
         <v>15</v>
       </c>
       <c r="I39" s="13" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="J39" s="13" t="s">
         <v>188</v>
@@ -10792,17 +10828,20 @@
         <v>2</v>
       </c>
       <c r="R39" s="24" t="s">
-        <v>677</v>
-      </c>
-      <c r="S39" s="29" t="s">
-        <v>809</v>
+        <v>873</v>
+      </c>
+      <c r="S39" s="28" t="s">
+        <v>799</v>
+      </c>
+      <c r="T39" s="38" t="s">
+        <v>877</v>
       </c>
       <c r="V39" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-010 Endpoints /projects/{id}/documents Sprint 3 Semana 4 2026-01-22 2026-01-22 1 P0 en curso API  CE-S2-001;CE-S3-006 Backend Lead Upload async status polling List/Get/Delete Bajo apps/api/src/routers/documents.py</v>
+        <v>CE-S4-010 Endpoints /projects/{id}/documents Sprint 3 Semana 4 2026-01-22 2026-01-22 1 P0 done API  CE-S2-001;CE-S3-006 Backend Lead Upload async status polling List/Get/Delete Bajo apps/api/src/routers/documents.py</v>
       </c>
       <c r="W39" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
     </row>
     <row r="40" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10855,18 +10894,18 @@
       <c r="Q40" s="13">
         <v>2</v>
       </c>
-      <c r="R40" s="35" t="s">
+      <c r="R40" s="32" t="s">
         <v>677</v>
       </c>
       <c r="S40" s="28" t="s">
-        <v>810</v>
+        <v>800</v>
       </c>
       <c r="V40" t="str">
         <f t="shared" si="0"/>
         <v>CE-S4-011 Script Rollback Automatizado Sprint 3 Semana 4 2026-01-21 2026-01-21 1 P0 done DevOps  Ninguna DevOps Rollback DB PITR + código git revert staging Medio scripts/rollback.sh</v>
       </c>
       <c r="W40" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
     </row>
     <row r="41" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10919,18 +10958,18 @@
       <c r="Q41" s="13">
         <v>2</v>
       </c>
-      <c r="R41" s="35" t="s">
+      <c r="R41" s="32" t="s">
         <v>677</v>
       </c>
       <c r="S41" s="28" t="s">
-        <v>811</v>
+        <v>801</v>
       </c>
       <c r="V41" t="str">
         <f t="shared" si="0"/>
         <v>CE-S4-012 Paginación Cursor-based Endpoints Sprint 3 Semana 4 2026-01-23 2026-01-23 1 P0 done API  CE-S3-008 Backend Lead Ningún endpoint &gt;100 items sin paginar Bajo apps/api/src/core/pagination.py</v>
       </c>
       <c r="W41" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
     </row>
     <row r="42" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -10983,18 +11022,18 @@
       <c r="Q42" s="13">
         <v>2</v>
       </c>
-      <c r="R42" s="35" t="s">
+      <c r="R42" s="32" t="s">
         <v>677</v>
       </c>
       <c r="S42" s="28" t="s">
-        <v>812</v>
+        <v>802</v>
       </c>
       <c r="V42" t="str">
         <f t="shared" si="0"/>
         <v>CE-S4-013 Optimizar Queries SQL EXPLAIN Sprint 3 Semana 4 2026-01-24 2026-01-24 1 P1 done Performance  Ninguna Backend Lead Queries lentas optimizadas 0 queries &gt;100ms Medio docs/performance/sql_optimization.md</v>
       </c>
       <c r="W42" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
     </row>
     <row r="43" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11047,18 +11086,18 @@
       <c r="Q43" s="13">
         <v>1</v>
       </c>
-      <c r="R43" s="37" t="s">
+      <c r="R43" s="34" t="s">
         <v>677</v>
       </c>
       <c r="S43" s="28" t="s">
-        <v>813</v>
+        <v>803</v>
       </c>
       <c r="V43" t="str">
         <f t="shared" si="0"/>
         <v>CE-S4-014 Índices Adicionales Búsqueda Sprint 3 Semana 4 2026-01-24 2026-01-24 0,5 P1 done Database  CE-S4-013 Backend Lead Índices campos filtro queries búsqueda &lt;50ms Bajo infrastructure/supabase/migrations/007_indexes.sql</v>
       </c>
       <c r="W43" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
     </row>
     <row r="44" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11087,7 +11126,7 @@
         <v>15</v>
       </c>
       <c r="I44" s="13" t="s">
-        <v>74</v>
+        <v>676</v>
       </c>
       <c r="J44" s="13" t="s">
         <v>145</v>
@@ -11113,15 +11152,18 @@
       <c r="Q44" s="13">
         <v>2</v>
       </c>
-      <c r="S44" s="24" t="s">
-        <v>814</v>
+      <c r="R44" s="34" t="s">
+        <v>678</v>
+      </c>
+      <c r="S44" s="28" t="s">
+        <v>878</v>
       </c>
       <c r="V44" t="str">
         <f t="shared" si="0"/>
-        <v>CE-S4-015 Tests Integración Coherence Engine Sprint 3 Semana 4 2026-01-24 2026-01-24 1 P0 Pendiente Testing Gate 5 CE-S4-005;CE-S2-015 QA Lead Tests proyectos golden 10 reglas correctas Medio tests/integration/coherence/</v>
+        <v>CE-S4-015 Tests Integración Coherence Engine Sprint 3 Semana 4 2026-01-24 2026-01-24 1 P0 done Testing Gate 5 CE-S4-005;CE-S2-015 QA Lead Tests proyectos golden 10 reglas correctas Medio tests/integration/coherence/</v>
       </c>
       <c r="W44" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
     </row>
     <row r="45" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11143,7 +11185,7 @@
       <c r="P45" s="13"/>
       <c r="Q45" s="13"/>
       <c r="S45" s="24" t="s">
-        <v>817</v>
+        <v>805</v>
       </c>
     </row>
     <row r="46" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11165,7 +11207,7 @@
       <c r="P46" s="13"/>
       <c r="Q46" s="13"/>
       <c r="S46" s="24" t="s">
-        <v>818</v>
+        <v>806</v>
       </c>
     </row>
     <row r="47" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11187,7 +11229,7 @@
       <c r="P47" s="13"/>
       <c r="Q47" s="13"/>
       <c r="S47" s="24" t="s">
-        <v>819</v>
+        <v>807</v>
       </c>
     </row>
     <row r="48" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11209,7 +11251,7 @@
       <c r="P48" s="13"/>
       <c r="Q48" s="13"/>
       <c r="S48" s="24" t="s">
-        <v>820</v>
+        <v>808</v>
       </c>
     </row>
     <row r="49" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11231,7 +11273,7 @@
       <c r="P49" s="13"/>
       <c r="Q49" s="13"/>
       <c r="S49" s="24" t="s">
-        <v>821</v>
+        <v>809</v>
       </c>
     </row>
     <row r="50" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11253,7 +11295,7 @@
       <c r="P50" s="13"/>
       <c r="Q50" s="13"/>
       <c r="S50" s="24" t="s">
-        <v>822</v>
+        <v>810</v>
       </c>
     </row>
     <row r="51" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11275,7 +11317,7 @@
       <c r="P51" s="13"/>
       <c r="Q51" s="13"/>
       <c r="S51" s="24" t="s">
-        <v>823</v>
+        <v>811</v>
       </c>
     </row>
     <row r="52" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11297,7 +11339,7 @@
       <c r="P52" s="13"/>
       <c r="Q52" s="13"/>
       <c r="S52" s="24" t="s">
-        <v>824</v>
+        <v>812</v>
       </c>
     </row>
     <row r="53" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11353,20 +11395,20 @@
         <v>5</v>
       </c>
       <c r="S53" s="24" t="s">
-        <v>815</v>
+        <v>874</v>
       </c>
       <c r="T53" s="24" t="s">
-        <v>816</v>
+        <v>804</v>
       </c>
       <c r="U53" s="24" t="s">
-        <v>826</v>
+        <v>814</v>
       </c>
       <c r="V53" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-001 StakeholderExtractorAgent Sprint 4 Semana 5 2026-01-27 2026-01-29 3 P0 Pendiente AI Gate 5 CE-S4-001 AI Lead Extracción NLP nombres/roles &gt;80% accuracy golden Alto apps/api/src/agents/stakeholder_extractor.py</v>
       </c>
       <c r="W53" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
     </row>
     <row r="54" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11422,14 +11464,14 @@
         <v>2</v>
       </c>
       <c r="S54" s="24" t="s">
-        <v>825</v>
+        <v>813</v>
       </c>
       <c r="V54" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-002 StakeholderClassifier Power/Interest Sprint 4 Semana 5 2026-01-28 2026-01-28 1 P0 Pendiente AI Gate 5 CE-S5-001 AI Lead Cuadrante asignado automáticamente 4 cuadrantes Medio apps/api/src/services/stakeholder_classifier.py</v>
       </c>
       <c r="W54" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
     </row>
     <row r="55" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11485,14 +11527,14 @@
         <v>5</v>
       </c>
       <c r="R55" s="24" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="V55" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-003 RACIGeneratorAgent Sprint 4 Semana 5 2026-01-29 2026-01-30 2 P0 Pendiente AI Gate 6 CE-S5-001;CE-S4-003 AI Lead Matriz RACI generada requires_review=True Alto apps/api/src/agents/raci_generator.py</v>
       </c>
       <c r="W55" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
     </row>
     <row r="56" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11514,7 +11556,7 @@
       <c r="P56" s="14"/>
       <c r="Q56" s="14"/>
       <c r="R56" s="24" t="s">
-        <v>827</v>
+        <v>815</v>
       </c>
     </row>
     <row r="57" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11538,7 +11580,7 @@
       <c r="P57" s="14"/>
       <c r="Q57" s="14"/>
       <c r="R57" s="28" t="s">
-        <v>844</v>
+        <v>832</v>
       </c>
     </row>
     <row r="58" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11562,7 +11604,7 @@
       <c r="P58" s="14"/>
       <c r="Q58" s="14"/>
       <c r="R58" s="28" t="s">
-        <v>845</v>
+        <v>833</v>
       </c>
     </row>
     <row r="59" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11582,14 +11624,14 @@
       <c r="N59" s="14"/>
       <c r="O59" s="14"/>
       <c r="P59" s="31" t="s">
-        <v>847</v>
+        <v>835</v>
       </c>
       <c r="Q59" s="14"/>
       <c r="R59" s="27" t="s">
-        <v>846</v>
+        <v>834</v>
       </c>
       <c r="S59" s="27" t="s">
-        <v>855</v>
+        <v>843</v>
       </c>
     </row>
     <row r="60" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11613,7 +11655,7 @@
       <c r="P60" s="14"/>
       <c r="Q60" s="14"/>
       <c r="R60" s="29" t="s">
-        <v>848</v>
+        <v>836</v>
       </c>
     </row>
     <row r="61" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11637,7 +11679,7 @@
       <c r="P61" s="14"/>
       <c r="Q61" s="14"/>
       <c r="R61" s="28" t="s">
-        <v>849</v>
+        <v>837</v>
       </c>
     </row>
     <row r="62" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11659,7 +11701,7 @@
       <c r="P62" s="14"/>
       <c r="Q62" s="14"/>
       <c r="R62" s="24" t="s">
-        <v>850</v>
+        <v>838</v>
       </c>
     </row>
     <row r="63" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11681,7 +11723,7 @@
       <c r="P63" s="14"/>
       <c r="Q63" s="14"/>
       <c r="R63" s="24" t="s">
-        <v>851</v>
+        <v>839</v>
       </c>
     </row>
     <row r="64" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11703,7 +11745,7 @@
       <c r="P64" s="14"/>
       <c r="Q64" s="14"/>
       <c r="R64" s="24" t="s">
-        <v>854</v>
+        <v>842</v>
       </c>
     </row>
     <row r="65" spans="1:23" x14ac:dyDescent="0.3">
@@ -11779,14 +11821,14 @@
         <v>3</v>
       </c>
       <c r="S66" s="24" t="s">
-        <v>828</v>
+        <v>816</v>
       </c>
       <c r="V66" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-004 Human-in-Loop Workflow Backend Sprint 4 Semana 5 2026-01-27 2026-01-28 2 P0 Pendiente Backend Gate 6 CE-S2-001 Backend Lead Endpoint aprobar/rechazar outputs agentes Alto apps/api/src/routers/approvals.py</v>
       </c>
       <c r="W66" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
     </row>
     <row r="67" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11842,14 +11884,14 @@
         <v>3</v>
       </c>
       <c r="S67" s="24" t="s">
-        <v>830</v>
+        <v>818</v>
       </c>
       <c r="V67" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-005 Knowledge Graph Básico NetworkX Sprint 4 Semana 5 2026-01-30 2026-01-31 2 P1 Pendiente Backend Gate 4 CE-S4-003 Backend Lead Nodos + edges queries multi-hop funcionan Medio apps/api/src/services/knowledge_graph.py</v>
       </c>
       <c r="W67" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
     </row>
     <row r="68" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11905,14 +11947,14 @@
         <v>3</v>
       </c>
       <c r="S68" s="24" t="s">
-        <v>831</v>
+        <v>819</v>
       </c>
       <c r="V68" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-006 Prompt Extracción Cláusulas Optimizado Sprint 4 Semana 5 2026-01-27 2026-01-28 2 P0 Pendiente AI Gate 5 CE-S2-008 AI Lead &gt;85% accuracy tipo/código/texto golden dataset Alto prompts/v1/clause_extraction.md</v>
       </c>
       <c r="W68" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
     </row>
     <row r="69" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -11968,17 +12010,17 @@
         <v>2</v>
       </c>
       <c r="S69" s="24" t="s">
-        <v>832</v>
+        <v>820</v>
       </c>
       <c r="T69" s="24" t="s">
-        <v>834</v>
+        <v>822</v>
       </c>
       <c r="V69" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-007 Prompt Clasificación Stakeholders Sprint 4 Semana 5 2026-01-29 2026-01-29 1 P0 Pendiente AI Gate 5 CE-S2-008 AI Lead &gt;80% accuracy clasificación poder/interés Medio prompts/v1/stakeholder_classification.md</v>
       </c>
       <c r="W69" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
     </row>
     <row r="70" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12034,20 +12076,20 @@
         <v>2</v>
       </c>
       <c r="S70" s="24" t="s">
-        <v>836</v>
+        <v>824</v>
       </c>
       <c r="T70" s="24" t="s">
-        <v>837</v>
+        <v>825</v>
       </c>
       <c r="U70" s="24" t="s">
-        <v>838</v>
+        <v>826</v>
       </c>
       <c r="V70" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-008 LlmRuleEvaluator Base Class Sprint 4 Semana 5 2026-01-28 2026-01-28 1 P0 Pendiente AI Gate 5 CE-S2-007 AI Lead Evaluador prompts reglas cualitativas interface Medio apps/api/src/coherence/llm_rule_evaluator.py</v>
       </c>
       <c r="W70" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
     </row>
     <row r="71" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12103,17 +12145,17 @@
         <v>3</v>
       </c>
       <c r="S71" s="24" t="s">
-        <v>839</v>
+        <v>827</v>
       </c>
       <c r="T71" s="24" t="s">
-        <v>840</v>
+        <v>828</v>
       </c>
       <c r="V71" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-009 Primera Regla LLM Cualitativa Sprint 4 Semana 5 2026-01-29 2026-01-30 2 P1 Pendiente AI Gate 5 CE-S5-008 AI Lead Regla detectar ambigüedades alcance evaluable Alto apps/api/src/coherence/rules/scope_ambiguity.py</v>
       </c>
       <c r="W71" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
     </row>
     <row r="72" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12169,14 +12211,14 @@
         <v>2</v>
       </c>
       <c r="S72" s="24" t="s">
-        <v>841</v>
+        <v>829</v>
       </c>
       <c r="V72" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-010 Endpoints /projects/{id}/stakeholders Sprint 4 Semana 5 2026-01-28 2026-01-28 1 P0 Pendiente API Gate 4 CE-S2-003 Backend Lead CRUD + clasificación source_clause_id Bajo apps/api/src/routers/stakeholders.py</v>
       </c>
       <c r="W72" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
     </row>
     <row r="73" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12232,14 +12274,14 @@
         <v>1</v>
       </c>
       <c r="S73" s="24" t="s">
-        <v>842</v>
+        <v>830</v>
       </c>
       <c r="V73" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-011 Endpoints /projects/{id}/raci Sprint 4 Semana 5 2026-01-29 2026-01-29 0,5 P0 Pendiente API Gate 6 CE-S2-003 Backend Lead Get matrix/Update human-in-loop flag Bajo apps/api/src/routers/raci.py</v>
       </c>
       <c r="W73" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
     </row>
     <row r="74" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12295,14 +12337,14 @@
         <v>3</v>
       </c>
       <c r="S74" s="24" t="s">
-        <v>852</v>
+        <v>840</v>
       </c>
       <c r="V74" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-012 Dashboard Observabilidad Básico Sprint 4 Semana 5 2026-01-27 2026-01-28 2 P0 Pendiente Frontend Gate 7 CE-S2-011 Frontend Lead Vista consumo tokens alertas automáticas budget Medio apps/web/src/pages/admin/observability.tsx</v>
       </c>
       <c r="W74" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
     </row>
     <row r="75" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12358,14 +12400,14 @@
         <v>2</v>
       </c>
       <c r="S75" s="24" t="s">
-        <v>853</v>
+        <v>841</v>
       </c>
       <c r="V75" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-013 Rate Limiting por Tenant Redis Sprint 4 Semana 5 2026-01-30 2026-01-30 1 P0 Pendiente Security Gate 7 CE-S2-004 Security Lead 60 req/min tenant 20 req/min user configurable Medio apps/api/src/middleware/rate_limiter.py</v>
       </c>
       <c r="W75" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
     </row>
     <row r="76" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12421,14 +12463,14 @@
         <v>2</v>
       </c>
       <c r="S76" s="24" t="s">
-        <v>856</v>
+        <v>844</v>
       </c>
       <c r="V76" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-014 Budget Alerts Email/Webhook Sprint 4 Semana 5 2026-01-31 2026-01-31 1 P0 Pendiente Backend Gate 7 CE-S4-002 Backend Lead Notificaciones admin 50/75/90/100% budget Medio apps/api/src/services/budget_alerts.py</v>
       </c>
       <c r="W76" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
     </row>
     <row r="77" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12484,14 +12526,14 @@
         <v>2</v>
       </c>
       <c r="S77" s="24" t="s">
-        <v>857</v>
+        <v>845</v>
       </c>
       <c r="V77" t="str">
         <f t="shared" si="0"/>
         <v>CE-S5-015 Tests Integración Stakeholder Flow Sprint 4 Semana 5 2026-01-31 2026-01-31 1 P0 Pendiente Testing Gate 5 CE-S5-001;CE-S5-003 QA Lead Extracción Clasificación RACI flujo completo Medio tests/integration/stakeholders/</v>
       </c>
       <c r="W77" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
     </row>
     <row r="78" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12547,14 +12589,14 @@
         <v>3</v>
       </c>
       <c r="S78" s="24" t="s">
-        <v>858</v>
+        <v>846</v>
       </c>
       <c r="V78" t="str">
         <f t="shared" si="0"/>
         <v>CE-S6-001 Vista Dashboard + Score Gauge Sprint 4 Semana 6 2026-02-02 2026-02-03 2 P0 Pendiente Frontend Gate 6 CE-S3-007 Frontend Lead Score 0-100 visual colores carga &lt;2s gauge animado Medio apps/web/src/pages/dashboard.tsx</v>
       </c>
       <c r="W78" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
     </row>
     <row r="79" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12608,17 +12650,17 @@
         <v>2</v>
       </c>
       <c r="S79" s="24" t="s">
-        <v>859</v>
+        <v>847</v>
       </c>
       <c r="T79" s="24" t="s">
-        <v>860</v>
+        <v>848</v>
       </c>
       <c r="V79" t="str">
         <f t="shared" si="0"/>
         <v>CE-S6-002 Vista Lista Proyectos Sprint 4 Semana 6 2026-02-02 2026-02-02 1 P0 Pendiente Frontend  CE-S3-008 Frontend Lead Filtros estado/búsqueda/orden paginación Bajo apps/web/src/pages/projects/index.tsx</v>
       </c>
       <c r="W79" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
     </row>
     <row r="80" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12674,14 +12716,14 @@
         <v>5</v>
       </c>
       <c r="S80" s="24" t="s">
-        <v>861</v>
+        <v>849</v>
       </c>
       <c r="V80" t="str">
         <f t="shared" si="0"/>
         <v>CE-S6-003 Evidence Viewer Links Cláusulas Sprint 4 Semana 6 2026-02-03 2026-02-04 2 P0 Pendiente Frontend Gate 4 CE-S4-009 Frontend Lead Click alerta cláusula WBS/BOM navegación bidireccional Alto apps/web/src/components/EvidenceViewer.tsx</v>
       </c>
       <c r="W80" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
     </row>
     <row r="81" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12735,14 +12777,14 @@
         <v>2</v>
       </c>
       <c r="S81" s="24" t="s">
-        <v>862</v>
+        <v>850</v>
       </c>
       <c r="V81" t="str">
         <f t="shared" si="0"/>
         <v>CE-S6-004 Panel Alertas Filtros Severidad Sprint 4 Semana 6 2026-02-04 2026-02-04 1 P0 Pendiente Frontend  CE-S6-003 Frontend Lead Vista alertas abiertas/resolved filtros bulk actions Bajo apps/web/src/pages/alerts.tsx</v>
       </c>
       <c r="W81" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
     </row>
     <row r="82" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12798,14 +12840,14 @@
         <v>3</v>
       </c>
       <c r="S82" s="24" t="s">
-        <v>863</v>
+        <v>851</v>
       </c>
       <c r="V82" t="str">
         <f t="shared" si="0"/>
         <v>CE-S6-005 Stakeholder Map Matriz Poder/Interés Sprint 4 Semana 6 2026-02-04 2026-02-05 2 P0 Pendiente Frontend Gate 6 CE-S5-010 Frontend Lead Visualización interactiva cuadrantes drag &amp; drop Medio apps/web/src/components/StakeholderMap.tsx</v>
       </c>
       <c r="W82" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
     </row>
     <row r="83" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12861,14 +12903,14 @@
         <v>2</v>
       </c>
       <c r="S83" s="24" t="s">
-        <v>864</v>
+        <v>852</v>
       </c>
       <c r="V83" t="str">
         <f t="shared" si="0"/>
         <v>CE-S6-006 RACI Viewer Editable Sprint 4 Semana 6 2026-02-05 2026-02-05 1 P0 Pendiente Frontend Gate 6 CE-S5-011 Frontend Lead Tabla WBS x Stakeholders RACI edición inline Medio apps/web/src/components/RACIViewer.tsx</v>
       </c>
       <c r="W83" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
     </row>
     <row r="84" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12924,14 +12966,14 @@
         <v>1</v>
       </c>
       <c r="S84" s="24" t="s">
-        <v>865</v>
+        <v>853</v>
       </c>
       <c r="V84" t="str">
         <f t="shared" si="0"/>
         <v>CE-S6-007 Modal Human-in-Loop Confirmación Sprint 4 Semana 6 2026-02-05 2026-02-05 0,5 P0 Pendiente Frontend Gate 6 CE-S5-004 Frontend Lead Confirmación aprobar/rechazar outputs IA workflow Medio apps/web/src/components/ApprovalModal.tsx</v>
       </c>
       <c r="W84" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
     </row>
     <row r="85" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -12987,17 +13029,17 @@
         <v>2</v>
       </c>
       <c r="S85" s="24" t="s">
-        <v>866</v>
+        <v>854</v>
       </c>
       <c r="T85" s="24" t="s">
-        <v>867</v>
+        <v>855</v>
       </c>
       <c r="V85" t="str">
         <f t="shared" ref="V85:V100" si="1">A85 &amp; " " &amp; B85 &amp; " " &amp; C85 &amp; " " &amp; D85 &amp; " " &amp; E85 &amp; " " &amp; F85 &amp; " " &amp; G85 &amp; " " &amp; H85 &amp; " " &amp; I85 &amp; " " &amp; J85 &amp; " " &amp; K85 &amp; " " &amp; L85 &amp; " " &amp; M85 &amp; " " &amp; N85 &amp; " " &amp; O85 &amp; " " &amp; P85</f>
         <v>CE-S6-008 Endpoints /projects/{id}/wbs y /bom Sprint 4 Semana 6 2026-02-02 2026-02-02 1 P0 Pendiente API Gate 4 CE-S2-003 Backend Lead CRUD WBS/BOM jerarquía WBS representada Bajo apps/api/src/routers/wbs.py</v>
       </c>
       <c r="W85" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
     </row>
     <row r="86" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -13051,14 +13093,14 @@
         <v>2</v>
       </c>
       <c r="S86" s="24" t="s">
-        <v>868</v>
+        <v>856</v>
       </c>
       <c r="V86" t="str">
         <f t="shared" si="1"/>
         <v>CE-S6-009 Endpoint POST /projects/{id}/analyze Sprint 4 Semana 6 2026-02-03 2026-02-03 1 P0 Pendiente API  CE-S3-006 Backend Lead Trigger análisis async retorna job_id polling Bajo apps/api/src/routers/analysis.py</v>
       </c>
       <c r="W86" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
     </row>
     <row r="87" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -13114,14 +13156,14 @@
         <v>2</v>
       </c>
       <c r="S87" s="24" t="s">
-        <v>869</v>
+        <v>857</v>
       </c>
       <c r="V87" t="str">
         <f t="shared" si="1"/>
         <v>CE-S6-010 Propagar clause_id a WBS Items Sprint 4 Semana 6 2026-02-02 2026-02-02 1 P0 Pendiente Backend Gate 4 CE-S3-005 Backend Lead funded_by_clause_id auto 100% WBS con FK Medio apps/api/src/services/wbs_service.py</v>
       </c>
       <c r="W87" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
     </row>
     <row r="88" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -13177,17 +13219,17 @@
         <v>2</v>
       </c>
       <c r="S88" s="24" t="s">
-        <v>870</v>
+        <v>858</v>
       </c>
       <c r="T88" s="24" t="s">
-        <v>871</v>
+        <v>859</v>
       </c>
       <c r="V88" t="str">
         <f t="shared" si="1"/>
         <v>CE-S6-011 Propagar clause_id a BOM Items Sprint 4 Semana 6 2026-02-03 2026-02-03 1 P0 Pendiente Backend Gate 4 CE-S3-005 Backend Lead contract_clause_id auto 100% BOM con FK Medio apps/api/src/services/bom_service.py</v>
       </c>
       <c r="W88" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
     </row>
     <row r="89" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -13243,14 +13285,14 @@
         <v>2</v>
       </c>
       <c r="S89" s="24" t="s">
-        <v>872</v>
+        <v>860</v>
       </c>
       <c r="V89" t="str">
         <f t="shared" si="1"/>
         <v>CE-S6-012 Evidence Viewer Logic Query Sprint 4 Semana 6 2026-02-04 2026-02-04 1 P0 Pendiente Backend Gate 4 CE-S6-010;CE-S6-011 Backend Lead Query reconstruye clause WBS BOM dado alert_id Medio apps/api/src/services/evidence_service.py</v>
       </c>
       <c r="W89" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
     </row>
     <row r="90" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -13304,14 +13346,14 @@
         <v>3</v>
       </c>
       <c r="S90" s="24" t="s">
-        <v>873</v>
+        <v>861</v>
       </c>
       <c r="V90" t="str">
         <f t="shared" si="1"/>
         <v>CE-S6-013 Graph RAG Service Abstracción Sprint 4 Semana 6 2026-02-03 2026-02-04 2 P1 Pendiente Backend  CE-S5-005 Backend Lead Interface GraphStore impl NetworkX tests mock Medio apps/api/src/services/graph_store.py</v>
       </c>
       <c r="W90" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
     </row>
     <row r="91" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -13367,14 +13409,14 @@
         <v>2</v>
       </c>
       <c r="S91" s="24" t="s">
-        <v>874</v>
+        <v>862</v>
       </c>
       <c r="V91" t="str">
         <f t="shared" si="1"/>
         <v>CE-S6-014 Circuit Breaker Claude API Sprint 4 Semana 6 2026-02-05 2026-02-05 1 P1 Pendiente Backend Gate 7 CE-S2-004 Backend Lead Retry backoff fallback caché API degradada ok Medio apps/api/src/ai/circuit_breaker.py</v>
       </c>
       <c r="W91" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
     </row>
     <row r="92" spans="1:23" ht="409.6" x14ac:dyDescent="0.3">
@@ -13428,14 +13470,14 @@
         <v>2</v>
       </c>
       <c r="S92" s="24" t="s">
-        <v>875</v>
+        <v>863</v>
       </c>
       <c r="V92" t="str">
         <f t="shared" si="1"/>
         <v>CE-S6-015 Async Processing Parsing Background Sprint 4 Semana 6 2026-02-05 2026-02-05 1 P0 Pendiente Backend  CE-S3-006 Backend Lead Parsing background polling status upload inmediato Bajo apps/api/src/tasks/parsing_tasks.py</v>
       </c>
       <c r="W92" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
     </row>
     <row r="93" spans="1:23" x14ac:dyDescent="0.3">
@@ -13495,7 +13537,7 @@
         <v>CE-S7-001 Cifrado Documentos R2 AES-256 Sprint 5 Semana 7 2026-02-09 2026-02-09 1 P0 Pendiente Security Gate 8 Ninguna Security Lead Server-side encryption keys tenant docs cifrados Alto apps/api/src/storage/encryption.py</v>
       </c>
       <c r="W93" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
     </row>
     <row r="94" spans="1:23" x14ac:dyDescent="0.3">
@@ -13555,7 +13597,7 @@
         <v>CE-S7-002 Política Retención Soft Delete Sprint 5 Semana 7 2026-02-09 2026-02-09 1 P0 Pendiente Security Gate 8 Ninguna Security Lead Soft delete hard delete 30 días job limpieza Medio apps/api/src/tasks/retention_job.py</v>
       </c>
       <c r="W94" t="s">
-        <v>787</v>
+        <v>783</v>
       </c>
     </row>
     <row r="95" spans="1:23" x14ac:dyDescent="0.3">
@@ -13615,7 +13657,7 @@
         <v>CE-S7-003 Auto-block Degradación Graceful Sprint 5 Semana 7 2026-02-10 2026-02-10 1 P0 Pendiente Backend Gate 7 CE-S4-002 Backend Lead Bloquear LLM 100% budget sistema sigue sin IA Alto apps/api/src/ai/budget_blocker.py</v>
       </c>
       <c r="W95" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
     </row>
     <row r="96" spans="1:23" x14ac:dyDescent="0.3">
@@ -13675,7 +13717,7 @@
         <v>CE-S7-004 Optimizar Prompts Reducir Tokens Sprint 5 Semana 7 2026-02-10 2026-02-11 2 P1 Pendiente AI Gate 7 CE-S2-008 AI Lead Few-shot reducido 20% reducción tokens promedio Medio prompts/v1/</v>
       </c>
       <c r="W96" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
     </row>
     <row r="97" spans="1:23" x14ac:dyDescent="0.3">
@@ -13735,7 +13777,7 @@
         <v>CE-S7-005 Dashboard Costes por Proyecto Sprint 5 Semana 7 2026-02-11 2026-02-11 1 P1 Pendiente Frontend Gate 7 CE-S5-012 Frontend Lead Breakdown costes operación/modelo coste real-time Bajo apps/web/src/components/CostDashboard.tsx</v>
       </c>
       <c r="W97" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
     </row>
     <row r="98" spans="1:23" x14ac:dyDescent="0.3">
@@ -13795,7 +13837,7 @@
         <v>CE-S7-006 Batch Processing Múltiples Docs Sprint 5 Semana 7 2026-02-11 2026-02-11 1 P1 Pendiente Backend Gate 7 CE-S3-006 Backend Lead 3 docs &lt;3x individual descuento contexto Medio apps/api/src/tasks/batch_processing.py</v>
       </c>
       <c r="W98" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
     </row>
     <row r="99" spans="1:23" x14ac:dyDescent="0.3">
@@ -13855,7 +13897,7 @@
         <v>CE-S7-007 Prompt Generación RACI Sprint 5 Semana 7 2026-02-10 2026-02-10 1 P1 Pendiente AI Gate 5 CE-S2-008 AI Lead Mapeo stakeholder WBS razonamiento RACI coherente Medio prompts/v1/raci_generation.md</v>
       </c>
       <c r="W99" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
     </row>
     <row r="100" spans="1:23" x14ac:dyDescent="0.3">
@@ -13913,7 +13955,7 @@
         <v>CE-S7-008 A/B Testing Prompts Framework Sprint 5 Semana 7 2026-02-12 2026-02-12 1 P2 Pendiente AI  CE-S2-008 AI Lead Framework comparar versiones métricas auto Bajo apps/api/src/ai/ab_testing.py</v>
       </c>
       <c r="W100" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
     </row>
     <row r="101" spans="1:23" x14ac:dyDescent="0.3">
@@ -14279,7 +14321,7 @@
         <v>2</v>
       </c>
       <c r="R107" s="24" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
     </row>
     <row r="108" spans="1:23" x14ac:dyDescent="0.3">
@@ -15748,16 +15790,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>615</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
@@ -16220,16 +16262,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>617</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
@@ -16972,16 +17014,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>619</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
@@ -17808,16 +17850,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>621</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
@@ -18544,16 +18586,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>623</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">

</xml_diff>